<commit_message>
add windows service and new data in database
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -530,6 +530,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+  </numFmts>
   <fonts count="35">
     <font>
       <sz val="11"/>
@@ -1475,6 +1478,350 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="24" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="24" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -1517,399 +1864,47 @@
     <xf numFmtId="0" fontId="34" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="24" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="24" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="10" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2018,6 +2013,14 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2057,7 +2060,7 @@
         <xdr:cNvPr id="13358" name="1 - Εικόνα" descr="Εικόνα που περιέχει έμβλημα, σύμβολο, οικόσημο, λογότυπο&#10;&#10;Περιγραφή που δημιουργήθηκε αυτόματα">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002E340000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00002E340000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2403,7 +2406,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2423,70 +2426,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A1" s="194"/>
-      <c r="B1" s="195"/>
-      <c r="C1" s="196"/>
-      <c r="D1" s="200" t="s">
+      <c r="A1" s="74"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="80" t="s">
         <v>109</v>
       </c>
-      <c r="E1" s="200"/>
-      <c r="F1" s="200"/>
-      <c r="G1" s="200"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A2" s="197"/>
-      <c r="B2" s="198"/>
-      <c r="C2" s="199"/>
-      <c r="D2" s="200"/>
-      <c r="E2" s="200"/>
-      <c r="F2" s="200"/>
-      <c r="G2" s="200"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
     </row>
     <row r="3" spans="1:7" ht="19.149999999999999" customHeight="1" thickBot="1">
-      <c r="A3" s="197"/>
-      <c r="B3" s="198"/>
-      <c r="C3" s="199"/>
-      <c r="D3" s="200"/>
-      <c r="E3" s="201"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="202" t="s">
+      <c r="A4" s="82" t="s">
         <v>110</v>
       </c>
-      <c r="B4" s="203"/>
-      <c r="C4" s="204"/>
-      <c r="D4" s="177" t="s">
+      <c r="B4" s="83"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="93" t="s">
         <v>111</v>
       </c>
-      <c r="E4" s="179"/>
-      <c r="F4" s="82" t="s">
+      <c r="E4" s="95"/>
+      <c r="F4" s="191" t="s">
         <v>112</v>
       </c>
-      <c r="G4" s="84"/>
+      <c r="G4" s="242"/>
     </row>
     <row r="5" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A5" s="205" t="s">
+      <c r="A5" s="85" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="206"/>
-      <c r="C5" s="207"/>
-      <c r="D5" s="178"/>
-      <c r="E5" s="180"/>
-      <c r="F5" s="83"/>
-      <c r="G5" s="85"/>
+      <c r="B5" s="86"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="96"/>
+      <c r="F5" s="192"/>
+      <c r="G5" s="243"/>
     </row>
     <row r="6" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A6" s="184" t="s">
+      <c r="A6" s="100" t="s">
         <v>142</v>
       </c>
-      <c r="B6" s="185"/>
-      <c r="C6" s="185"/>
-      <c r="D6" s="186"/>
-      <c r="E6" s="187"/>
-      <c r="F6" s="187"/>
-      <c r="G6" s="188"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="F6" s="103"/>
+      <c r="G6" s="104"/>
     </row>
     <row r="7" spans="1:7" ht="15.75" thickBot="1"/>
     <row r="8" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
@@ -2501,127 +2504,127 @@
       <c r="G8" s="45"/>
     </row>
     <row r="9" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A9" s="176" t="s">
+      <c r="A9" s="88" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="176"/>
-      <c r="C9" s="176"/>
-      <c r="D9" s="176"/>
-      <c r="E9" s="181"/>
-      <c r="F9" s="181"/>
-      <c r="G9" s="181"/>
+      <c r="B9" s="88"/>
+      <c r="C9" s="88"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="89"/>
+      <c r="F9" s="89"/>
+      <c r="G9" s="89"/>
     </row>
     <row r="10" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A10" s="182" t="s">
+      <c r="A10" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="182"/>
-      <c r="C10" s="182"/>
-      <c r="D10" s="182"/>
-      <c r="E10" s="181"/>
-      <c r="F10" s="181"/>
-      <c r="G10" s="181"/>
+      <c r="B10" s="72"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="89"/>
+      <c r="F10" s="89"/>
+      <c r="G10" s="89"/>
     </row>
     <row r="11" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A11" s="176" t="s">
+      <c r="A11" s="88" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="176"/>
-      <c r="C11" s="176"/>
-      <c r="D11" s="176"/>
-      <c r="E11" s="191"/>
-      <c r="F11" s="192"/>
-      <c r="G11" s="193"/>
+      <c r="B11" s="88"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="90"/>
+      <c r="F11" s="91"/>
+      <c r="G11" s="92"/>
     </row>
     <row r="12" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A12" s="182" t="s">
+      <c r="A12" s="72" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="182"/>
-      <c r="C12" s="182"/>
-      <c r="D12" s="182"/>
-      <c r="E12" s="183"/>
-      <c r="F12" s="183"/>
-      <c r="G12" s="183"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="73"/>
+      <c r="G12" s="73"/>
     </row>
     <row r="13" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A13" s="176" t="s">
+      <c r="A13" s="88" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="176"/>
-      <c r="C13" s="176"/>
-      <c r="D13" s="176"/>
-      <c r="E13" s="191"/>
-      <c r="F13" s="192"/>
-      <c r="G13" s="193"/>
+      <c r="B13" s="88"/>
+      <c r="C13" s="88"/>
+      <c r="D13" s="88"/>
+      <c r="E13" s="90"/>
+      <c r="F13" s="91"/>
+      <c r="G13" s="92"/>
     </row>
     <row r="14" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A14" s="182" t="s">
+      <c r="A14" s="72" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="182"/>
-      <c r="C14" s="182"/>
-      <c r="D14" s="182"/>
-      <c r="E14" s="183"/>
-      <c r="F14" s="183"/>
-      <c r="G14" s="183"/>
+      <c r="B14" s="72"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
+      <c r="G14" s="73"/>
     </row>
     <row r="15" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A15" s="176" t="s">
+      <c r="A15" s="88" t="s">
         <v>121</v>
       </c>
-      <c r="B15" s="176"/>
-      <c r="C15" s="176"/>
-      <c r="D15" s="176"/>
-      <c r="E15" s="181"/>
-      <c r="F15" s="181"/>
-      <c r="G15" s="181"/>
+      <c r="B15" s="88"/>
+      <c r="C15" s="88"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="89"/>
     </row>
     <row r="16" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A16" s="182" t="s">
+      <c r="A16" s="72" t="s">
         <v>122</v>
       </c>
-      <c r="B16" s="182"/>
-      <c r="C16" s="182"/>
-      <c r="D16" s="182"/>
-      <c r="E16" s="183"/>
-      <c r="F16" s="183"/>
-      <c r="G16" s="183"/>
+      <c r="B16" s="72"/>
+      <c r="C16" s="72"/>
+      <c r="D16" s="72"/>
+      <c r="E16" s="73"/>
+      <c r="F16" s="73"/>
+      <c r="G16" s="73"/>
     </row>
     <row r="17" spans="1:7" ht="49.5" customHeight="1" thickBot="1">
-      <c r="A17" s="176" t="s">
+      <c r="A17" s="88" t="s">
         <v>123</v>
       </c>
-      <c r="B17" s="176"/>
-      <c r="C17" s="176"/>
-      <c r="D17" s="176"/>
-      <c r="E17" s="189"/>
-      <c r="F17" s="181"/>
-      <c r="G17" s="181"/>
+      <c r="B17" s="88"/>
+      <c r="C17" s="88"/>
+      <c r="D17" s="88"/>
+      <c r="E17" s="105"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
     </row>
     <row r="19" spans="1:7" hidden="1"/>
     <row r="20" spans="1:7" ht="26.25">
-      <c r="A20" s="127" t="s">
+      <c r="A20" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="127"/>
-      <c r="C20" s="127"/>
-      <c r="D20" s="127"/>
-      <c r="E20" s="127"/>
-      <c r="F20" s="127"/>
-      <c r="G20" s="127"/>
+      <c r="B20" s="106"/>
+      <c r="C20" s="106"/>
+      <c r="D20" s="106"/>
+      <c r="E20" s="106"/>
+      <c r="F20" s="106"/>
+      <c r="G20" s="106"/>
     </row>
     <row r="21" spans="1:7" ht="63">
       <c r="A21" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="170" t="s">
+      <c r="B21" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="C21" s="171"/>
-      <c r="D21" s="171"/>
-      <c r="E21" s="171"/>
-      <c r="F21" s="172"/>
+      <c r="C21" s="108"/>
+      <c r="D21" s="108"/>
+      <c r="E21" s="108"/>
+      <c r="F21" s="109"/>
       <c r="G21" s="47" t="s">
         <v>3</v>
       </c>
@@ -2630,13 +2633,13 @@
       <c r="A22" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="96" t="s">
+      <c r="B22" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="96"/>
-      <c r="D22" s="96"/>
-      <c r="E22" s="96"/>
-      <c r="F22" s="96"/>
+      <c r="C22" s="110"/>
+      <c r="D22" s="110"/>
+      <c r="E22" s="110"/>
+      <c r="F22" s="110"/>
       <c r="G22" s="42">
         <v>0</v>
       </c>
@@ -2645,13 +2648,13 @@
       <c r="A23" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="190" t="s">
+      <c r="B23" s="111" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="190"/>
-      <c r="D23" s="190"/>
-      <c r="E23" s="190"/>
-      <c r="F23" s="190"/>
+      <c r="C23" s="111"/>
+      <c r="D23" s="111"/>
+      <c r="E23" s="111"/>
+      <c r="F23" s="111"/>
       <c r="G23" s="5">
         <v>8</v>
       </c>
@@ -2660,13 +2663,13 @@
       <c r="A24" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="96" t="s">
+      <c r="B24" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="96"/>
-      <c r="D24" s="96"/>
-      <c r="E24" s="96"/>
-      <c r="F24" s="96"/>
+      <c r="C24" s="110"/>
+      <c r="D24" s="110"/>
+      <c r="E24" s="110"/>
+      <c r="F24" s="110"/>
       <c r="G24" s="42">
         <v>4</v>
       </c>
@@ -2675,13 +2678,13 @@
       <c r="A25" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="190" t="s">
+      <c r="B25" s="111" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="190"/>
-      <c r="D25" s="190"/>
-      <c r="E25" s="190"/>
-      <c r="F25" s="190"/>
+      <c r="C25" s="111"/>
+      <c r="D25" s="111"/>
+      <c r="E25" s="111"/>
+      <c r="F25" s="111"/>
       <c r="G25" s="5">
         <v>12</v>
       </c>
@@ -2690,13 +2693,13 @@
       <c r="A26" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="133" t="s">
+      <c r="B26" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="133"/>
-      <c r="D26" s="133"/>
-      <c r="E26" s="133"/>
-      <c r="F26" s="133"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
+      <c r="E26" s="112"/>
+      <c r="F26" s="112"/>
       <c r="G26" s="42">
         <v>12</v>
       </c>
@@ -2705,54 +2708,54 @@
       <c r="A27" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="169" t="s">
+      <c r="B27" s="97" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="169"/>
-      <c r="D27" s="169"/>
-      <c r="E27" s="169"/>
-      <c r="F27" s="169"/>
+      <c r="C27" s="97"/>
+      <c r="D27" s="97"/>
+      <c r="E27" s="97"/>
+      <c r="F27" s="97"/>
       <c r="G27" s="5">
         <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="38.25" customHeight="1">
-      <c r="A28" s="173" t="s">
+      <c r="A28" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="174"/>
-      <c r="C28" s="174"/>
-      <c r="D28" s="174"/>
-      <c r="E28" s="174"/>
-      <c r="F28" s="175"/>
+      <c r="B28" s="115"/>
+      <c r="C28" s="115"/>
+      <c r="D28" s="115"/>
+      <c r="E28" s="115"/>
+      <c r="F28" s="116"/>
       <c r="G28" s="41" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A29" s="107" t="s">
+      <c r="A29" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="107"/>
-      <c r="C29" s="107"/>
-      <c r="D29" s="107"/>
-      <c r="E29" s="107"/>
-      <c r="F29" s="107"/>
+      <c r="B29" s="98"/>
+      <c r="C29" s="98"/>
+      <c r="D29" s="98"/>
+      <c r="E29" s="98"/>
+      <c r="F29" s="98"/>
       <c r="G29" s="55">
         <f>VLOOKUP(A29,A22:G27,7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="26.25">
-      <c r="A31" s="127" t="s">
+      <c r="A31" s="106" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="127"/>
-      <c r="C31" s="127"/>
-      <c r="D31" s="127"/>
-      <c r="E31" s="127"/>
-      <c r="F31" s="127"/>
-      <c r="G31" s="127"/>
+      <c r="B31" s="106"/>
+      <c r="C31" s="106"/>
+      <c r="D31" s="106"/>
+      <c r="E31" s="106"/>
+      <c r="F31" s="106"/>
+      <c r="G31" s="106"/>
     </row>
     <row r="32" spans="1:7" ht="45">
       <c r="A32" s="51" t="s">
@@ -2761,12 +2764,12 @@
       <c r="B32" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="C32" s="170" t="s">
+      <c r="C32" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="171"/>
-      <c r="E32" s="171"/>
-      <c r="F32" s="172"/>
+      <c r="D32" s="108"/>
+      <c r="E32" s="108"/>
+      <c r="F32" s="109"/>
       <c r="G32" s="49" t="s">
         <v>3</v>
       </c>
@@ -2778,12 +2781,12 @@
       <c r="B33" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="133" t="s">
+      <c r="C33" s="112" t="s">
         <v>22</v>
       </c>
-      <c r="D33" s="133"/>
-      <c r="E33" s="133"/>
-      <c r="F33" s="133"/>
+      <c r="D33" s="112"/>
+      <c r="E33" s="112"/>
+      <c r="F33" s="112"/>
       <c r="G33" s="42">
         <v>0</v>
       </c>
@@ -2795,12 +2798,12 @@
       <c r="B34" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="169" t="s">
+      <c r="C34" s="97" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="169"/>
-      <c r="E34" s="169"/>
-      <c r="F34" s="169"/>
+      <c r="D34" s="97"/>
+      <c r="E34" s="97"/>
+      <c r="F34" s="97"/>
       <c r="G34" s="5">
         <v>4</v>
       </c>
@@ -2812,12 +2815,12 @@
       <c r="B35" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="133" t="s">
+      <c r="C35" s="112" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="133"/>
-      <c r="E35" s="133"/>
-      <c r="F35" s="133"/>
+      <c r="D35" s="112"/>
+      <c r="E35" s="112"/>
+      <c r="F35" s="112"/>
       <c r="G35" s="42">
         <v>8</v>
       </c>
@@ -2829,142 +2832,142 @@
       <c r="B36" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="169" t="s">
+      <c r="C36" s="97" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="169"/>
-      <c r="E36" s="169"/>
-      <c r="F36" s="169"/>
+      <c r="D36" s="97"/>
+      <c r="E36" s="97"/>
+      <c r="F36" s="97"/>
       <c r="G36" s="5">
         <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="42.75" customHeight="1">
-      <c r="A37" s="131" t="s">
+      <c r="A37" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="131"/>
-      <c r="C37" s="131"/>
-      <c r="D37" s="131"/>
-      <c r="E37" s="131"/>
-      <c r="F37" s="131"/>
+      <c r="B37" s="99"/>
+      <c r="C37" s="99"/>
+      <c r="D37" s="99"/>
+      <c r="E37" s="99"/>
+      <c r="F37" s="99"/>
       <c r="G37" s="41" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A38" s="107">
+      <c r="A38" s="98">
         <v>1</v>
       </c>
-      <c r="B38" s="107"/>
-      <c r="C38" s="107"/>
-      <c r="D38" s="107"/>
-      <c r="E38" s="107"/>
-      <c r="F38" s="107"/>
+      <c r="B38" s="98"/>
+      <c r="C38" s="98"/>
+      <c r="D38" s="98"/>
+      <c r="E38" s="98"/>
+      <c r="F38" s="98"/>
       <c r="G38" s="55">
         <f>VLOOKUP(A38,A33:G36,7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="30">
-      <c r="A41" s="145" t="s">
+      <c r="A41" s="113" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="145"/>
-      <c r="C41" s="145"/>
-      <c r="D41" s="145"/>
-      <c r="E41" s="145"/>
-      <c r="F41" s="145"/>
-      <c r="G41" s="145"/>
+      <c r="B41" s="113"/>
+      <c r="C41" s="113"/>
+      <c r="D41" s="113"/>
+      <c r="E41" s="113"/>
+      <c r="F41" s="113"/>
+      <c r="G41" s="113"/>
     </row>
     <row r="42" spans="1:7" ht="30">
-      <c r="A42" s="163" t="s">
+      <c r="A42" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="B42" s="163"/>
-      <c r="C42" s="163"/>
-      <c r="D42" s="157" t="s">
+      <c r="B42" s="123"/>
+      <c r="C42" s="123"/>
+      <c r="D42" s="117" t="s">
         <v>29</v>
       </c>
-      <c r="E42" s="157"/>
-      <c r="F42" s="157"/>
+      <c r="E42" s="117"/>
+      <c r="F42" s="117"/>
       <c r="G42" s="48" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15" customHeight="1">
-      <c r="A43" s="164">
+      <c r="A43" s="124">
         <f>SUM(G29,G38)</f>
         <v>0</v>
       </c>
-      <c r="B43" s="164"/>
-      <c r="C43" s="164"/>
+      <c r="B43" s="124"/>
+      <c r="C43" s="124"/>
       <c r="D43" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E43" s="168" t="s">
+      <c r="E43" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="F43" s="168"/>
+      <c r="F43" s="128"/>
       <c r="G43" s="42" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15" customHeight="1">
-      <c r="A44" s="164"/>
-      <c r="B44" s="164"/>
-      <c r="C44" s="164"/>
+      <c r="A44" s="124"/>
+      <c r="B44" s="124"/>
+      <c r="C44" s="124"/>
       <c r="D44" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E44" s="168" t="s">
+      <c r="E44" s="128" t="s">
         <v>35</v>
       </c>
-      <c r="F44" s="168"/>
-      <c r="G44" s="165" t="s">
+      <c r="F44" s="128"/>
+      <c r="G44" s="125" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15" customHeight="1">
-      <c r="A45" s="164"/>
-      <c r="B45" s="164"/>
-      <c r="C45" s="164"/>
+      <c r="A45" s="124"/>
+      <c r="B45" s="124"/>
+      <c r="C45" s="124"/>
       <c r="D45" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E45" s="168" t="s">
+      <c r="E45" s="128" t="s">
         <v>36</v>
       </c>
-      <c r="F45" s="168"/>
-      <c r="G45" s="166"/>
+      <c r="F45" s="128"/>
+      <c r="G45" s="126"/>
     </row>
     <row r="46" spans="1:7" ht="44.25" customHeight="1">
-      <c r="A46" s="160" t="s">
+      <c r="A46" s="120" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="161"/>
-      <c r="C46" s="161"/>
-      <c r="D46" s="162"/>
-      <c r="E46" s="158" t="str">
+      <c r="B46" s="121"/>
+      <c r="C46" s="121"/>
+      <c r="D46" s="122"/>
+      <c r="E46" s="118" t="str">
         <f>IF(A43&lt;=8,E43,IF(AND(A43&gt;=9,A43&lt;=18),E44,E45))</f>
         <v>Χαμηλό</v>
       </c>
-      <c r="F46" s="159"/>
+      <c r="F46" s="119"/>
       <c r="G46" s="57" t="str">
         <f>IF(A43&gt;8,G44,G43)</f>
         <v>ΌΧΙ*</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="41.25" customHeight="1">
-      <c r="A47" s="167" t="s">
+      <c r="A47" s="127" t="s">
         <v>125</v>
       </c>
-      <c r="B47" s="167"/>
-      <c r="C47" s="167"/>
-      <c r="D47" s="167"/>
-      <c r="E47" s="167"/>
-      <c r="F47" s="167"/>
-      <c r="G47" s="167"/>
+      <c r="B47" s="127"/>
+      <c r="C47" s="127"/>
+      <c r="D47" s="127"/>
+      <c r="E47" s="127"/>
+      <c r="F47" s="127"/>
+      <c r="G47" s="127"/>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="44"/>
@@ -2976,139 +2979,139 @@
       <c r="G48" s="44"/>
     </row>
     <row r="50" spans="1:7" ht="24">
-      <c r="A50" s="110" t="s">
+      <c r="A50" s="165" t="s">
         <v>138</v>
       </c>
-      <c r="B50" s="110"/>
-      <c r="C50" s="110"/>
-      <c r="D50" s="110"/>
-      <c r="E50" s="110"/>
-      <c r="F50" s="110"/>
-      <c r="G50" s="110"/>
+      <c r="B50" s="165"/>
+      <c r="C50" s="165"/>
+      <c r="D50" s="165"/>
+      <c r="E50" s="165"/>
+      <c r="F50" s="165"/>
+      <c r="G50" s="165"/>
     </row>
     <row r="51" spans="1:7" ht="26.25">
-      <c r="A51" s="127" t="s">
+      <c r="A51" s="106" t="s">
         <v>40</v>
       </c>
-      <c r="B51" s="127"/>
-      <c r="C51" s="127"/>
-      <c r="D51" s="127"/>
-      <c r="E51" s="127"/>
-      <c r="F51" s="127"/>
-      <c r="G51" s="127"/>
+      <c r="B51" s="106"/>
+      <c r="C51" s="106"/>
+      <c r="D51" s="106"/>
+      <c r="E51" s="106"/>
+      <c r="F51" s="106"/>
+      <c r="G51" s="106"/>
     </row>
     <row r="52" spans="1:7" ht="15.75">
-      <c r="A52" s="156" t="s">
+      <c r="A52" s="138" t="s">
         <v>41</v>
       </c>
-      <c r="B52" s="156"/>
-      <c r="C52" s="156" t="s">
+      <c r="B52" s="138"/>
+      <c r="C52" s="138" t="s">
         <v>45</v>
       </c>
-      <c r="D52" s="156"/>
-      <c r="E52" s="156"/>
-      <c r="F52" s="156"/>
+      <c r="D52" s="138"/>
+      <c r="E52" s="138"/>
+      <c r="F52" s="138"/>
       <c r="G52" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:7">
-      <c r="A53" s="96" t="s">
+      <c r="A53" s="110" t="s">
         <v>126</v>
       </c>
-      <c r="B53" s="96"/>
-      <c r="C53" s="96" t="s">
+      <c r="B53" s="110"/>
+      <c r="C53" s="110" t="s">
         <v>126</v>
       </c>
-      <c r="D53" s="96"/>
-      <c r="E53" s="96"/>
-      <c r="F53" s="96"/>
+      <c r="D53" s="110"/>
+      <c r="E53" s="110"/>
+      <c r="F53" s="110"/>
       <c r="G53" s="42" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="54" spans="1:7">
-      <c r="A54" s="96" t="s">
+      <c r="A54" s="110" t="s">
         <v>42</v>
       </c>
-      <c r="B54" s="96"/>
-      <c r="C54" s="96" t="s">
+      <c r="B54" s="110"/>
+      <c r="C54" s="110" t="s">
         <v>46</v>
       </c>
-      <c r="D54" s="96"/>
-      <c r="E54" s="96"/>
-      <c r="F54" s="96"/>
+      <c r="D54" s="110"/>
+      <c r="E54" s="110"/>
+      <c r="F54" s="110"/>
       <c r="G54" s="42">
         <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:7">
-      <c r="A55" s="155" t="s">
+      <c r="A55" s="137" t="s">
         <v>35</v>
       </c>
-      <c r="B55" s="155"/>
-      <c r="C55" s="155" t="s">
+      <c r="B55" s="137"/>
+      <c r="C55" s="137" t="s">
         <v>47</v>
       </c>
-      <c r="D55" s="155"/>
-      <c r="E55" s="155"/>
-      <c r="F55" s="155"/>
+      <c r="D55" s="137"/>
+      <c r="E55" s="137"/>
+      <c r="F55" s="137"/>
       <c r="G55" s="13">
         <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:7">
-      <c r="A56" s="96" t="s">
+      <c r="A56" s="110" t="s">
         <v>43</v>
       </c>
-      <c r="B56" s="96"/>
-      <c r="C56" s="96" t="s">
+      <c r="B56" s="110"/>
+      <c r="C56" s="110" t="s">
         <v>48</v>
       </c>
-      <c r="D56" s="96"/>
-      <c r="E56" s="96"/>
-      <c r="F56" s="96"/>
+      <c r="D56" s="110"/>
+      <c r="E56" s="110"/>
+      <c r="F56" s="110"/>
       <c r="G56" s="42">
         <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:7">
-      <c r="A57" s="155" t="s">
+      <c r="A57" s="137" t="s">
         <v>44</v>
       </c>
-      <c r="B57" s="155"/>
-      <c r="C57" s="155" t="s">
+      <c r="B57" s="137"/>
+      <c r="C57" s="137" t="s">
         <v>49</v>
       </c>
-      <c r="D57" s="155"/>
-      <c r="E57" s="155"/>
-      <c r="F57" s="155"/>
+      <c r="D57" s="137"/>
+      <c r="E57" s="137"/>
+      <c r="F57" s="137"/>
       <c r="G57" s="13">
         <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="18" customHeight="1">
-      <c r="A58" s="131" t="s">
+      <c r="A58" s="99" t="s">
         <v>64</v>
       </c>
-      <c r="B58" s="131"/>
-      <c r="C58" s="131"/>
-      <c r="D58" s="131"/>
-      <c r="E58" s="131"/>
-      <c r="F58" s="131"/>
+      <c r="B58" s="99"/>
+      <c r="C58" s="99"/>
+      <c r="D58" s="99"/>
+      <c r="E58" s="99"/>
+      <c r="F58" s="99"/>
       <c r="G58" s="41" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A59" s="107" t="s">
+      <c r="A59" s="98" t="s">
         <v>42</v>
       </c>
-      <c r="B59" s="107"/>
-      <c r="C59" s="107"/>
-      <c r="D59" s="107"/>
-      <c r="E59" s="107"/>
-      <c r="F59" s="107"/>
+      <c r="B59" s="98"/>
+      <c r="C59" s="98"/>
+      <c r="D59" s="98"/>
+      <c r="E59" s="98"/>
+      <c r="F59" s="98"/>
       <c r="G59" s="55">
         <f>VLOOKUP(A59,A53:G57,7,FALSE)</f>
         <v>0</v>
@@ -3116,27 +3119,27 @@
     </row>
     <row r="60" spans="1:7" ht="59.25" customHeight="1"/>
     <row r="61" spans="1:7" ht="26.25">
-      <c r="A61" s="127" t="s">
+      <c r="A61" s="106" t="s">
         <v>76</v>
       </c>
-      <c r="B61" s="127"/>
-      <c r="C61" s="127"/>
-      <c r="D61" s="127"/>
-      <c r="E61" s="127"/>
-      <c r="F61" s="127"/>
-      <c r="G61" s="127"/>
+      <c r="B61" s="106"/>
+      <c r="C61" s="106"/>
+      <c r="D61" s="106"/>
+      <c r="E61" s="106"/>
+      <c r="F61" s="106"/>
+      <c r="G61" s="106"/>
     </row>
     <row r="62" spans="1:7" ht="31.5">
       <c r="A62" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="B62" s="146" t="s">
+      <c r="B62" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="C62" s="147"/>
-      <c r="D62" s="147"/>
-      <c r="E62" s="147"/>
-      <c r="F62" s="148"/>
+      <c r="C62" s="134"/>
+      <c r="D62" s="134"/>
+      <c r="E62" s="134"/>
+      <c r="F62" s="135"/>
       <c r="G62" s="54" t="s">
         <v>3</v>
       </c>
@@ -3145,13 +3148,13 @@
       <c r="A63" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="B63" s="111" t="s">
+      <c r="B63" s="166" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="112"/>
-      <c r="D63" s="112"/>
-      <c r="E63" s="112"/>
-      <c r="F63" s="113"/>
+      <c r="C63" s="167"/>
+      <c r="D63" s="167"/>
+      <c r="E63" s="167"/>
+      <c r="F63" s="168"/>
       <c r="G63" s="14" t="s">
         <v>126</v>
       </c>
@@ -3160,13 +3163,13 @@
       <c r="A64" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="B64" s="133" t="s">
+      <c r="B64" s="112" t="s">
         <v>52</v>
       </c>
-      <c r="C64" s="133"/>
-      <c r="D64" s="133"/>
-      <c r="E64" s="133"/>
-      <c r="F64" s="133"/>
+      <c r="C64" s="112"/>
+      <c r="D64" s="112"/>
+      <c r="E64" s="112"/>
+      <c r="F64" s="112"/>
       <c r="G64" s="42">
         <v>0</v>
       </c>
@@ -3175,13 +3178,13 @@
       <c r="A65" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B65" s="149" t="s">
+      <c r="B65" s="136" t="s">
         <v>53</v>
       </c>
-      <c r="C65" s="149"/>
-      <c r="D65" s="149"/>
-      <c r="E65" s="149"/>
-      <c r="F65" s="149"/>
+      <c r="C65" s="136"/>
+      <c r="D65" s="136"/>
+      <c r="E65" s="136"/>
+      <c r="F65" s="136"/>
       <c r="G65" s="13">
         <v>4</v>
       </c>
@@ -3190,54 +3193,54 @@
       <c r="A66" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="B66" s="133" t="s">
+      <c r="B66" s="112" t="s">
         <v>54</v>
       </c>
-      <c r="C66" s="133"/>
-      <c r="D66" s="133"/>
-      <c r="E66" s="133"/>
-      <c r="F66" s="133"/>
+      <c r="C66" s="112"/>
+      <c r="D66" s="112"/>
+      <c r="E66" s="112"/>
+      <c r="F66" s="112"/>
       <c r="G66" s="42">
         <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="41.25" customHeight="1">
-      <c r="A67" s="151" t="s">
+      <c r="A67" s="129" t="s">
         <v>65</v>
       </c>
-      <c r="B67" s="152"/>
-      <c r="C67" s="152"/>
-      <c r="D67" s="152"/>
-      <c r="E67" s="152"/>
-      <c r="F67" s="153"/>
+      <c r="B67" s="130"/>
+      <c r="C67" s="130"/>
+      <c r="D67" s="130"/>
+      <c r="E67" s="130"/>
+      <c r="F67" s="131"/>
       <c r="G67" s="50" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="68" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A68" s="107" t="s">
+      <c r="A68" s="98" t="s">
         <v>50</v>
       </c>
-      <c r="B68" s="107"/>
-      <c r="C68" s="107"/>
-      <c r="D68" s="107"/>
-      <c r="E68" s="107"/>
-      <c r="F68" s="107"/>
+      <c r="B68" s="98"/>
+      <c r="C68" s="98"/>
+      <c r="D68" s="98"/>
+      <c r="E68" s="98"/>
+      <c r="F68" s="98"/>
       <c r="G68" s="55">
         <f>VLOOKUP(A68,A63:G66,7,FALSE)</f>
         <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="27.75">
-      <c r="A71" s="154" t="s">
+      <c r="A71" s="132" t="s">
         <v>75</v>
       </c>
-      <c r="B71" s="154"/>
-      <c r="C71" s="154"/>
-      <c r="D71" s="154"/>
-      <c r="E71" s="154"/>
-      <c r="F71" s="154"/>
-      <c r="G71" s="154"/>
+      <c r="B71" s="132"/>
+      <c r="C71" s="132"/>
+      <c r="D71" s="132"/>
+      <c r="E71" s="132"/>
+      <c r="F71" s="132"/>
+      <c r="G71" s="132"/>
     </row>
     <row r="72" spans="1:7" ht="51">
       <c r="A72" s="53" t="s">
@@ -3246,12 +3249,12 @@
       <c r="B72" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="C72" s="146" t="s">
+      <c r="C72" s="133" t="s">
         <v>60</v>
       </c>
-      <c r="D72" s="147"/>
-      <c r="E72" s="147"/>
-      <c r="F72" s="148"/>
+      <c r="D72" s="134"/>
+      <c r="E72" s="134"/>
+      <c r="F72" s="135"/>
       <c r="G72" s="54" t="s">
         <v>3</v>
       </c>
@@ -3263,12 +3266,12 @@
       <c r="B73" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="C73" s="111" t="s">
+      <c r="C73" s="166" t="s">
         <v>126</v>
       </c>
-      <c r="D73" s="112"/>
-      <c r="E73" s="112"/>
-      <c r="F73" s="113"/>
+      <c r="D73" s="167"/>
+      <c r="E73" s="167"/>
+      <c r="F73" s="168"/>
       <c r="G73" s="14" t="s">
         <v>126</v>
       </c>
@@ -3280,12 +3283,12 @@
       <c r="B74" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C74" s="133" t="s">
+      <c r="C74" s="112" t="s">
         <v>61</v>
       </c>
-      <c r="D74" s="133"/>
-      <c r="E74" s="133"/>
-      <c r="F74" s="133"/>
+      <c r="D74" s="112"/>
+      <c r="E74" s="112"/>
+      <c r="F74" s="112"/>
       <c r="G74" s="42">
         <v>0</v>
       </c>
@@ -3297,12 +3300,12 @@
       <c r="B75" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C75" s="149" t="s">
+      <c r="C75" s="136" t="s">
         <v>62</v>
       </c>
-      <c r="D75" s="149"/>
-      <c r="E75" s="149"/>
-      <c r="F75" s="149"/>
+      <c r="D75" s="136"/>
+      <c r="E75" s="136"/>
+      <c r="F75" s="136"/>
       <c r="G75" s="13">
         <v>4</v>
       </c>
@@ -3314,38 +3317,38 @@
       <c r="B76" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C76" s="133" t="s">
+      <c r="C76" s="112" t="s">
         <v>63</v>
       </c>
-      <c r="D76" s="133"/>
-      <c r="E76" s="133"/>
-      <c r="F76" s="133"/>
+      <c r="D76" s="112"/>
+      <c r="E76" s="112"/>
+      <c r="F76" s="112"/>
       <c r="G76" s="42">
         <v>6</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="39" customHeight="1">
-      <c r="A77" s="150" t="s">
+      <c r="A77" s="151" t="s">
         <v>66</v>
       </c>
-      <c r="B77" s="150"/>
-      <c r="C77" s="150"/>
-      <c r="D77" s="150"/>
-      <c r="E77" s="150"/>
-      <c r="F77" s="150"/>
+      <c r="B77" s="151"/>
+      <c r="C77" s="151"/>
+      <c r="D77" s="151"/>
+      <c r="E77" s="151"/>
+      <c r="F77" s="151"/>
       <c r="G77" s="43" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="78" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A78" s="107">
+      <c r="A78" s="98">
         <v>2</v>
       </c>
-      <c r="B78" s="107"/>
-      <c r="C78" s="107"/>
-      <c r="D78" s="107"/>
-      <c r="E78" s="107"/>
-      <c r="F78" s="107"/>
+      <c r="B78" s="98"/>
+      <c r="C78" s="98"/>
+      <c r="D78" s="98"/>
+      <c r="E78" s="98"/>
+      <c r="F78" s="98"/>
       <c r="G78" s="55">
         <f>VLOOKUP(A78,A73:G76,7)</f>
         <v>4</v>
@@ -3353,38 +3356,38 @@
     </row>
     <row r="80" spans="1:7" hidden="1"/>
     <row r="81" spans="1:7" ht="30">
-      <c r="A81" s="145" t="s">
+      <c r="A81" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="B81" s="145"/>
-      <c r="C81" s="145"/>
-      <c r="D81" s="145"/>
-      <c r="E81" s="145"/>
-      <c r="F81" s="145"/>
-      <c r="G81" s="145"/>
+      <c r="B81" s="113"/>
+      <c r="C81" s="113"/>
+      <c r="D81" s="113"/>
+      <c r="E81" s="113"/>
+      <c r="F81" s="113"/>
+      <c r="G81" s="113"/>
     </row>
     <row r="82" spans="1:7" ht="42" customHeight="1">
-      <c r="A82" s="87" t="s">
+      <c r="A82" s="139" t="s">
         <v>67</v>
       </c>
-      <c r="B82" s="87"/>
-      <c r="C82" s="87"/>
-      <c r="D82" s="87"/>
-      <c r="E82" s="87"/>
-      <c r="F82" s="87" t="s">
+      <c r="B82" s="139"/>
+      <c r="C82" s="139"/>
+      <c r="D82" s="139"/>
+      <c r="E82" s="139"/>
+      <c r="F82" s="139" t="s">
         <v>131</v>
       </c>
-      <c r="G82" s="87"/>
+      <c r="G82" s="139"/>
     </row>
     <row r="83" spans="1:7" ht="15" customHeight="1">
-      <c r="A83" s="136">
+      <c r="A83" s="142">
         <f>SUM(G29,G38,G59,G68,G78)</f>
         <v>4</v>
       </c>
-      <c r="B83" s="137"/>
-      <c r="C83" s="137"/>
-      <c r="D83" s="137"/>
-      <c r="E83" s="138"/>
+      <c r="B83" s="143"/>
+      <c r="C83" s="143"/>
+      <c r="D83" s="143"/>
+      <c r="E83" s="144"/>
       <c r="F83" s="12" t="s">
         <v>68</v>
       </c>
@@ -3393,11 +3396,11 @@
       </c>
     </row>
     <row r="84" spans="1:7" ht="15" customHeight="1">
-      <c r="A84" s="139"/>
-      <c r="B84" s="140"/>
-      <c r="C84" s="140"/>
-      <c r="D84" s="140"/>
-      <c r="E84" s="141"/>
+      <c r="A84" s="145"/>
+      <c r="B84" s="146"/>
+      <c r="C84" s="146"/>
+      <c r="D84" s="146"/>
+      <c r="E84" s="147"/>
       <c r="F84" s="19" t="s">
         <v>69</v>
       </c>
@@ -3406,11 +3409,11 @@
       </c>
     </row>
     <row r="85" spans="1:7" ht="15" customHeight="1">
-      <c r="A85" s="142"/>
-      <c r="B85" s="143"/>
-      <c r="C85" s="143"/>
-      <c r="D85" s="143"/>
-      <c r="E85" s="144"/>
+      <c r="A85" s="148"/>
+      <c r="B85" s="149"/>
+      <c r="C85" s="149"/>
+      <c r="D85" s="149"/>
+      <c r="E85" s="150"/>
       <c r="F85" s="12" t="s">
         <v>70</v>
       </c>
@@ -3419,436 +3422,436 @@
       </c>
     </row>
     <row r="86" spans="1:7" ht="44.25" customHeight="1">
-      <c r="A86" s="95" t="s">
+      <c r="A86" s="141" t="s">
         <v>72</v>
       </c>
-      <c r="B86" s="95"/>
-      <c r="C86" s="95"/>
-      <c r="D86" s="95"/>
-      <c r="E86" s="95"/>
-      <c r="F86" s="135" t="str">
+      <c r="B86" s="141"/>
+      <c r="C86" s="141"/>
+      <c r="D86" s="141"/>
+      <c r="E86" s="141"/>
+      <c r="F86" s="140" t="str">
         <f>IF(A83="-","-",IF(A83&lt;=14,G83,IF(AND(A83&gt;=15,A83&lt;=30),G84,G85)))</f>
         <v>Χαμηλό</v>
       </c>
-      <c r="G86" s="135"/>
+      <c r="G86" s="140"/>
     </row>
     <row r="89" spans="1:7" ht="26.25">
-      <c r="A89" s="127" t="s">
+      <c r="A89" s="106" t="s">
         <v>108</v>
       </c>
-      <c r="B89" s="127"/>
-      <c r="C89" s="127"/>
-      <c r="D89" s="127"/>
-      <c r="E89" s="127"/>
-      <c r="F89" s="127"/>
-      <c r="G89" s="127"/>
+      <c r="B89" s="106"/>
+      <c r="C89" s="106"/>
+      <c r="D89" s="106"/>
+      <c r="E89" s="106"/>
+      <c r="F89" s="106"/>
+      <c r="G89" s="106"/>
     </row>
     <row r="90" spans="1:7">
-      <c r="A90" s="128" t="s">
+      <c r="A90" s="152" t="s">
         <v>127</v>
       </c>
-      <c r="B90" s="128"/>
-      <c r="C90" s="128"/>
-      <c r="D90" s="128"/>
-      <c r="E90" s="128" t="s">
+      <c r="B90" s="152"/>
+      <c r="C90" s="152"/>
+      <c r="D90" s="152"/>
+      <c r="E90" s="152" t="s">
         <v>103</v>
       </c>
-      <c r="F90" s="128"/>
-      <c r="G90" s="128"/>
+      <c r="F90" s="152"/>
+      <c r="G90" s="152"/>
     </row>
     <row r="91" spans="1:7">
-      <c r="A91" s="97" t="s">
+      <c r="A91" s="156" t="s">
         <v>126</v>
       </c>
-      <c r="B91" s="98"/>
-      <c r="C91" s="98"/>
-      <c r="D91" s="99"/>
-      <c r="E91" s="97" t="s">
+      <c r="B91" s="157"/>
+      <c r="C91" s="157"/>
+      <c r="D91" s="158"/>
+      <c r="E91" s="156" t="s">
         <v>126</v>
       </c>
-      <c r="F91" s="98"/>
-      <c r="G91" s="99"/>
+      <c r="F91" s="157"/>
+      <c r="G91" s="158"/>
     </row>
     <row r="92" spans="1:7">
-      <c r="A92" s="96" t="s">
+      <c r="A92" s="110" t="s">
         <v>34</v>
       </c>
-      <c r="B92" s="96"/>
-      <c r="C92" s="96"/>
-      <c r="D92" s="96"/>
-      <c r="E92" s="96" t="s">
+      <c r="B92" s="110"/>
+      <c r="C92" s="110"/>
+      <c r="D92" s="110"/>
+      <c r="E92" s="110" t="s">
         <v>132</v>
       </c>
-      <c r="F92" s="96"/>
-      <c r="G92" s="96"/>
+      <c r="F92" s="110"/>
+      <c r="G92" s="110"/>
     </row>
     <row r="93" spans="1:7">
-      <c r="A93" s="129" t="s">
+      <c r="A93" s="153" t="s">
         <v>35</v>
       </c>
-      <c r="B93" s="129"/>
-      <c r="C93" s="129"/>
-      <c r="D93" s="129"/>
-      <c r="E93" s="129" t="s">
+      <c r="B93" s="153"/>
+      <c r="C93" s="153"/>
+      <c r="D93" s="153"/>
+      <c r="E93" s="153" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="129"/>
-      <c r="G93" s="129"/>
+      <c r="F93" s="153"/>
+      <c r="G93" s="153"/>
     </row>
     <row r="94" spans="1:7">
-      <c r="A94" s="133" t="s">
+      <c r="A94" s="112" t="s">
         <v>36</v>
       </c>
-      <c r="B94" s="133"/>
-      <c r="C94" s="133"/>
-      <c r="D94" s="133"/>
-      <c r="E94" s="96" t="s">
+      <c r="B94" s="112"/>
+      <c r="C94" s="112"/>
+      <c r="D94" s="112"/>
+      <c r="E94" s="110" t="s">
         <v>106</v>
       </c>
-      <c r="F94" s="96"/>
-      <c r="G94" s="96"/>
+      <c r="F94" s="110"/>
+      <c r="G94" s="110"/>
     </row>
     <row r="95" spans="1:7" ht="15.75">
-      <c r="A95" s="130" t="s">
+      <c r="A95" s="154" t="s">
         <v>107</v>
       </c>
-      <c r="B95" s="130"/>
-      <c r="C95" s="130"/>
-      <c r="D95" s="130"/>
-      <c r="E95" s="130"/>
-      <c r="F95" s="130"/>
-      <c r="G95" s="130"/>
+      <c r="B95" s="154"/>
+      <c r="C95" s="154"/>
+      <c r="D95" s="154"/>
+      <c r="E95" s="154"/>
+      <c r="F95" s="154"/>
+      <c r="G95" s="154"/>
     </row>
     <row r="96" spans="1:7" ht="37.5" customHeight="1">
-      <c r="A96" s="131" t="s">
+      <c r="A96" s="99" t="s">
         <v>129</v>
       </c>
-      <c r="B96" s="131"/>
-      <c r="C96" s="131"/>
-      <c r="D96" s="131"/>
-      <c r="E96" s="125" t="s">
+      <c r="B96" s="99"/>
+      <c r="C96" s="99"/>
+      <c r="D96" s="99"/>
+      <c r="E96" s="161" t="s">
         <v>103</v>
       </c>
-      <c r="F96" s="125"/>
-      <c r="G96" s="125"/>
+      <c r="F96" s="161"/>
+      <c r="G96" s="161"/>
     </row>
     <row r="97" spans="1:7" ht="55.5" customHeight="1">
-      <c r="A97" s="134" t="str">
+      <c r="A97" s="155" t="str">
         <f>F86</f>
         <v>Χαμηλό</v>
       </c>
-      <c r="B97" s="134"/>
-      <c r="C97" s="134"/>
-      <c r="D97" s="134"/>
-      <c r="E97" s="132" t="str">
+      <c r="B97" s="155"/>
+      <c r="C97" s="155"/>
+      <c r="D97" s="155"/>
+      <c r="E97" s="162" t="str">
         <f>VLOOKUP(A97,A91:G94,5,FALSE)</f>
         <v>Δεν πραγματοποιούνται έλεγχοι</v>
       </c>
-      <c r="F97" s="132"/>
-      <c r="G97" s="132"/>
+      <c r="F97" s="162"/>
+      <c r="G97" s="162"/>
     </row>
     <row r="100" spans="1:7" ht="24">
-      <c r="A100" s="110" t="s">
+      <c r="A100" s="165" t="s">
         <v>134</v>
       </c>
-      <c r="B100" s="110"/>
-      <c r="C100" s="110"/>
-      <c r="D100" s="110"/>
-      <c r="E100" s="110"/>
-      <c r="F100" s="110"/>
-      <c r="G100" s="110"/>
+      <c r="B100" s="165"/>
+      <c r="C100" s="165"/>
+      <c r="D100" s="165"/>
+      <c r="E100" s="165"/>
+      <c r="F100" s="165"/>
+      <c r="G100" s="165"/>
     </row>
     <row r="101" spans="1:7" ht="26.25">
-      <c r="A101" s="127" t="s">
+      <c r="A101" s="106" t="s">
         <v>73</v>
       </c>
-      <c r="B101" s="127"/>
-      <c r="C101" s="127"/>
-      <c r="D101" s="127"/>
-      <c r="E101" s="127"/>
-      <c r="F101" s="127"/>
-      <c r="G101" s="127"/>
+      <c r="B101" s="106"/>
+      <c r="C101" s="106"/>
+      <c r="D101" s="106"/>
+      <c r="E101" s="106"/>
+      <c r="F101" s="106"/>
+      <c r="G101" s="106"/>
     </row>
     <row r="102" spans="1:7" ht="24.75" customHeight="1">
-      <c r="A102" s="100" t="s">
+      <c r="A102" s="159" t="s">
         <v>71</v>
       </c>
-      <c r="B102" s="100"/>
-      <c r="C102" s="100"/>
-      <c r="D102" s="100"/>
-      <c r="E102" s="100"/>
-      <c r="F102" s="100"/>
+      <c r="B102" s="159"/>
+      <c r="C102" s="159"/>
+      <c r="D102" s="159"/>
+      <c r="E102" s="159"/>
+      <c r="F102" s="159"/>
       <c r="G102" s="26" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="15.75">
-      <c r="A103" s="100" t="s">
+      <c r="A103" s="159" t="s">
         <v>126</v>
       </c>
-      <c r="B103" s="100"/>
-      <c r="C103" s="100"/>
-      <c r="D103" s="100"/>
-      <c r="E103" s="100"/>
-      <c r="F103" s="100"/>
+      <c r="B103" s="159"/>
+      <c r="C103" s="159"/>
+      <c r="D103" s="159"/>
+      <c r="E103" s="159"/>
+      <c r="F103" s="159"/>
       <c r="G103" s="26" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="104" spans="1:7">
-      <c r="A104" s="96" t="s">
+      <c r="A104" s="110" t="s">
         <v>50</v>
       </c>
-      <c r="B104" s="96"/>
-      <c r="C104" s="96"/>
-      <c r="D104" s="96"/>
-      <c r="E104" s="96"/>
-      <c r="F104" s="96"/>
+      <c r="B104" s="110"/>
+      <c r="C104" s="110"/>
+      <c r="D104" s="110"/>
+      <c r="E104" s="110"/>
+      <c r="F104" s="110"/>
       <c r="G104" s="42">
         <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:7">
-      <c r="A105" s="101" t="s">
+      <c r="A105" s="160" t="s">
         <v>55</v>
       </c>
-      <c r="B105" s="101"/>
-      <c r="C105" s="101"/>
-      <c r="D105" s="101"/>
-      <c r="E105" s="101"/>
-      <c r="F105" s="101"/>
+      <c r="B105" s="160"/>
+      <c r="C105" s="160"/>
+      <c r="D105" s="160"/>
+      <c r="E105" s="160"/>
+      <c r="F105" s="160"/>
       <c r="G105" s="24">
         <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:7">
-      <c r="A106" s="96" t="s">
+      <c r="A106" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="B106" s="96"/>
-      <c r="C106" s="96"/>
-      <c r="D106" s="96"/>
-      <c r="E106" s="96"/>
-      <c r="F106" s="96"/>
+      <c r="B106" s="110"/>
+      <c r="C106" s="110"/>
+      <c r="D106" s="110"/>
+      <c r="E106" s="110"/>
+      <c r="F106" s="110"/>
       <c r="G106" s="42">
         <v>12</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="47.25" customHeight="1">
-      <c r="A107" s="106" t="s">
+      <c r="A107" s="205" t="s">
         <v>81</v>
       </c>
-      <c r="B107" s="106"/>
-      <c r="C107" s="106"/>
-      <c r="D107" s="106"/>
-      <c r="E107" s="106"/>
-      <c r="F107" s="106"/>
+      <c r="B107" s="205"/>
+      <c r="C107" s="205"/>
+      <c r="D107" s="205"/>
+      <c r="E107" s="205"/>
+      <c r="F107" s="205"/>
       <c r="G107" s="27" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="33.75">
-      <c r="A108" s="107" t="s">
+      <c r="A108" s="98" t="s">
         <v>126</v>
       </c>
-      <c r="B108" s="107"/>
-      <c r="C108" s="107"/>
-      <c r="D108" s="107"/>
-      <c r="E108" s="107"/>
-      <c r="F108" s="107"/>
+      <c r="B108" s="98"/>
+      <c r="C108" s="98"/>
+      <c r="D108" s="98"/>
+      <c r="E108" s="98"/>
+      <c r="F108" s="98"/>
       <c r="G108" s="40" t="str">
         <f>VLOOKUP(A108,A103:G106,7,FALSE)</f>
         <v>-</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="26.25">
-      <c r="A112" s="127" t="s">
+      <c r="A112" s="106" t="s">
         <v>77</v>
       </c>
-      <c r="B112" s="127"/>
-      <c r="C112" s="127"/>
-      <c r="D112" s="127"/>
-      <c r="E112" s="127"/>
-      <c r="F112" s="127"/>
-      <c r="G112" s="127"/>
+      <c r="B112" s="106"/>
+      <c r="C112" s="106"/>
+      <c r="D112" s="106"/>
+      <c r="E112" s="106"/>
+      <c r="F112" s="106"/>
+      <c r="G112" s="106"/>
     </row>
     <row r="113" spans="1:7" ht="27.75" customHeight="1">
-      <c r="A113" s="100" t="s">
+      <c r="A113" s="159" t="s">
         <v>77</v>
       </c>
-      <c r="B113" s="100"/>
-      <c r="C113" s="100"/>
-      <c r="D113" s="100"/>
-      <c r="E113" s="100"/>
-      <c r="F113" s="100"/>
+      <c r="B113" s="159"/>
+      <c r="C113" s="159"/>
+      <c r="D113" s="159"/>
+      <c r="E113" s="159"/>
+      <c r="F113" s="159"/>
       <c r="G113" s="26" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="15.75">
-      <c r="A114" s="100" t="s">
+      <c r="A114" s="159" t="s">
         <v>126</v>
       </c>
-      <c r="B114" s="100"/>
-      <c r="C114" s="100"/>
-      <c r="D114" s="100"/>
-      <c r="E114" s="100"/>
-      <c r="F114" s="100"/>
+      <c r="B114" s="159"/>
+      <c r="C114" s="159"/>
+      <c r="D114" s="159"/>
+      <c r="E114" s="159"/>
+      <c r="F114" s="159"/>
       <c r="G114" s="26" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="115" spans="1:7">
-      <c r="A115" s="96" t="s">
+      <c r="A115" s="110" t="s">
         <v>78</v>
       </c>
-      <c r="B115" s="96"/>
-      <c r="C115" s="96"/>
-      <c r="D115" s="96"/>
-      <c r="E115" s="96"/>
-      <c r="F115" s="96"/>
+      <c r="B115" s="110"/>
+      <c r="C115" s="110"/>
+      <c r="D115" s="110"/>
+      <c r="E115" s="110"/>
+      <c r="F115" s="110"/>
       <c r="G115" s="42">
         <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:7">
-      <c r="A116" s="101" t="s">
+      <c r="A116" s="160" t="s">
         <v>79</v>
       </c>
-      <c r="B116" s="101"/>
-      <c r="C116" s="101"/>
-      <c r="D116" s="101"/>
-      <c r="E116" s="101"/>
-      <c r="F116" s="101"/>
+      <c r="B116" s="160"/>
+      <c r="C116" s="160"/>
+      <c r="D116" s="160"/>
+      <c r="E116" s="160"/>
+      <c r="F116" s="160"/>
       <c r="G116" s="24">
         <v>3</v>
       </c>
     </row>
     <row r="117" spans="1:7">
-      <c r="A117" s="96" t="s">
+      <c r="A117" s="110" t="s">
         <v>80</v>
       </c>
-      <c r="B117" s="96"/>
-      <c r="C117" s="96"/>
-      <c r="D117" s="96"/>
-      <c r="E117" s="96"/>
-      <c r="F117" s="96"/>
+      <c r="B117" s="110"/>
+      <c r="C117" s="110"/>
+      <c r="D117" s="110"/>
+      <c r="E117" s="110"/>
+      <c r="F117" s="110"/>
       <c r="G117" s="42">
         <v>6</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="18">
-      <c r="A118" s="102" t="s">
+      <c r="A118" s="201" t="s">
         <v>82</v>
       </c>
-      <c r="B118" s="102"/>
-      <c r="C118" s="102"/>
-      <c r="D118" s="102"/>
-      <c r="E118" s="102"/>
-      <c r="F118" s="102"/>
+      <c r="B118" s="201"/>
+      <c r="C118" s="201"/>
+      <c r="D118" s="201"/>
+      <c r="E118" s="201"/>
+      <c r="F118" s="201"/>
       <c r="G118" s="27" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="26.25">
-      <c r="A119" s="103" t="s">
+      <c r="A119" s="202" t="s">
         <v>126</v>
       </c>
-      <c r="B119" s="104"/>
-      <c r="C119" s="104"/>
-      <c r="D119" s="104"/>
-      <c r="E119" s="104"/>
-      <c r="F119" s="105"/>
+      <c r="B119" s="203"/>
+      <c r="C119" s="203"/>
+      <c r="D119" s="203"/>
+      <c r="E119" s="203"/>
+      <c r="F119" s="204"/>
       <c r="G119" s="55" t="str">
         <f>VLOOKUP(A119,A114:G117,7,FALSE)</f>
         <v>-</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="35.25" customHeight="1">
-      <c r="A122" s="86" t="s">
+      <c r="A122" s="193" t="s">
         <v>84</v>
       </c>
-      <c r="B122" s="86"/>
-      <c r="C122" s="86"/>
-      <c r="D122" s="86"/>
-      <c r="E122" s="86"/>
-      <c r="F122" s="86"/>
-      <c r="G122" s="86"/>
+      <c r="B122" s="193"/>
+      <c r="C122" s="193"/>
+      <c r="D122" s="193"/>
+      <c r="E122" s="193"/>
+      <c r="F122" s="193"/>
+      <c r="G122" s="193"/>
     </row>
     <row r="123" spans="1:7" ht="135" customHeight="1">
-      <c r="A123" s="87" t="s">
+      <c r="A123" s="139" t="s">
         <v>140</v>
       </c>
-      <c r="B123" s="87"/>
-      <c r="C123" s="87"/>
+      <c r="B123" s="139"/>
+      <c r="C123" s="139"/>
       <c r="D123" s="65" t="s">
         <v>94</v>
       </c>
-      <c r="E123" s="87" t="s">
+      <c r="E123" s="139" t="s">
         <v>85</v>
       </c>
-      <c r="F123" s="87"/>
+      <c r="F123" s="139"/>
       <c r="G123" s="59" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="15" customHeight="1">
-      <c r="A124" s="94" t="str">
+      <c r="A124" s="200" t="str">
         <f>IF(AND(G108="-",G119="-"),"-",IF(G119="-",SUM(A83,G108),SUM(A83,G108,G119)))</f>
         <v>-</v>
       </c>
-      <c r="B124" s="94"/>
-      <c r="C124" s="94"/>
+      <c r="B124" s="200"/>
+      <c r="C124" s="200"/>
       <c r="D124" s="63" t="s">
         <v>89</v>
       </c>
-      <c r="E124" s="88" t="s">
+      <c r="E124" s="194" t="s">
         <v>86</v>
       </c>
-      <c r="F124" s="89"/>
+      <c r="F124" s="195"/>
       <c r="G124" s="29" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="15" customHeight="1">
-      <c r="A125" s="94"/>
-      <c r="B125" s="94"/>
-      <c r="C125" s="94"/>
+      <c r="A125" s="200"/>
+      <c r="B125" s="200"/>
+      <c r="C125" s="200"/>
       <c r="D125" s="64" t="s">
         <v>90</v>
       </c>
-      <c r="E125" s="90" t="s">
+      <c r="E125" s="196" t="s">
         <v>87</v>
       </c>
-      <c r="F125" s="91"/>
+      <c r="F125" s="197"/>
       <c r="G125" s="31" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="15" customHeight="1">
-      <c r="A126" s="94"/>
-      <c r="B126" s="94"/>
-      <c r="C126" s="94"/>
+      <c r="A126" s="200"/>
+      <c r="B126" s="200"/>
+      <c r="C126" s="200"/>
       <c r="D126" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="E126" s="92" t="s">
+      <c r="E126" s="198" t="s">
         <v>88</v>
       </c>
-      <c r="F126" s="93"/>
+      <c r="F126" s="199"/>
       <c r="G126" s="29" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="53.25" customHeight="1">
-      <c r="A127" s="95" t="s">
+      <c r="A127" s="141" t="s">
         <v>93</v>
       </c>
-      <c r="B127" s="95"/>
-      <c r="C127" s="95"/>
-      <c r="D127" s="95"/>
-      <c r="E127" s="95"/>
-      <c r="F127" s="95"/>
+      <c r="B127" s="141"/>
+      <c r="C127" s="141"/>
+      <c r="D127" s="141"/>
+      <c r="E127" s="141"/>
+      <c r="F127" s="141"/>
       <c r="G127" s="62" t="str">
         <f>IF(A124="-","-",IF(G119="-",IF(A124&lt;=19,G124,IF(A124&gt;=40,G126,G125)),IF(A124&lt;=21,G124,IF(A124&gt;=44,G126,G125))))</f>
         <v>-</v>
@@ -3864,173 +3867,173 @@
       <c r="G128" s="61"/>
     </row>
     <row r="131" spans="1:7" ht="26.25">
-      <c r="A131" s="127" t="s">
+      <c r="A131" s="106" t="s">
         <v>139</v>
       </c>
-      <c r="B131" s="127"/>
-      <c r="C131" s="127"/>
-      <c r="D131" s="127"/>
-      <c r="E131" s="127"/>
-      <c r="F131" s="127"/>
-      <c r="G131" s="127"/>
+      <c r="B131" s="106"/>
+      <c r="C131" s="106"/>
+      <c r="D131" s="106"/>
+      <c r="E131" s="106"/>
+      <c r="F131" s="106"/>
+      <c r="G131" s="106"/>
     </row>
     <row r="132" spans="1:7">
-      <c r="A132" s="128" t="s">
+      <c r="A132" s="152" t="s">
         <v>128</v>
       </c>
-      <c r="B132" s="128"/>
-      <c r="C132" s="128"/>
-      <c r="D132" s="128"/>
-      <c r="E132" s="128" t="s">
+      <c r="B132" s="152"/>
+      <c r="C132" s="152"/>
+      <c r="D132" s="152"/>
+      <c r="E132" s="152" t="s">
         <v>103</v>
       </c>
-      <c r="F132" s="128"/>
-      <c r="G132" s="128"/>
+      <c r="F132" s="152"/>
+      <c r="G132" s="152"/>
     </row>
     <row r="133" spans="1:7">
-      <c r="A133" s="97" t="s">
+      <c r="A133" s="156" t="s">
         <v>126</v>
       </c>
-      <c r="B133" s="98"/>
-      <c r="C133" s="98"/>
-      <c r="D133" s="99"/>
-      <c r="E133" s="97" t="s">
+      <c r="B133" s="157"/>
+      <c r="C133" s="157"/>
+      <c r="D133" s="158"/>
+      <c r="E133" s="156" t="s">
         <v>126</v>
       </c>
-      <c r="F133" s="98"/>
-      <c r="G133" s="99"/>
+      <c r="F133" s="157"/>
+      <c r="G133" s="158"/>
     </row>
     <row r="134" spans="1:7">
-      <c r="A134" s="96" t="s">
+      <c r="A134" s="110" t="s">
         <v>34</v>
       </c>
-      <c r="B134" s="96"/>
-      <c r="C134" s="96"/>
-      <c r="D134" s="96"/>
-      <c r="E134" s="96" t="s">
+      <c r="B134" s="110"/>
+      <c r="C134" s="110"/>
+      <c r="D134" s="110"/>
+      <c r="E134" s="110" t="s">
         <v>104</v>
       </c>
-      <c r="F134" s="96"/>
-      <c r="G134" s="96"/>
+      <c r="F134" s="110"/>
+      <c r="G134" s="110"/>
     </row>
     <row r="135" spans="1:7">
-      <c r="A135" s="129" t="s">
+      <c r="A135" s="153" t="s">
         <v>35</v>
       </c>
-      <c r="B135" s="129"/>
-      <c r="C135" s="129"/>
-      <c r="D135" s="129"/>
-      <c r="E135" s="129" t="s">
+      <c r="B135" s="153"/>
+      <c r="C135" s="153"/>
+      <c r="D135" s="153"/>
+      <c r="E135" s="153" t="s">
         <v>105</v>
       </c>
-      <c r="F135" s="129"/>
-      <c r="G135" s="129"/>
+      <c r="F135" s="153"/>
+      <c r="G135" s="153"/>
     </row>
     <row r="136" spans="1:7">
-      <c r="A136" s="96" t="s">
+      <c r="A136" s="110" t="s">
         <v>36</v>
       </c>
-      <c r="B136" s="96"/>
-      <c r="C136" s="96"/>
-      <c r="D136" s="96"/>
-      <c r="E136" s="96" t="s">
+      <c r="B136" s="110"/>
+      <c r="C136" s="110"/>
+      <c r="D136" s="110"/>
+      <c r="E136" s="110" t="s">
         <v>106</v>
       </c>
-      <c r="F136" s="96"/>
-      <c r="G136" s="96"/>
+      <c r="F136" s="110"/>
+      <c r="G136" s="110"/>
     </row>
     <row r="137" spans="1:7" ht="15.75">
-      <c r="A137" s="130" t="s">
+      <c r="A137" s="154" t="s">
         <v>107</v>
       </c>
-      <c r="B137" s="130"/>
-      <c r="C137" s="130"/>
-      <c r="D137" s="130"/>
-      <c r="E137" s="130"/>
-      <c r="F137" s="130"/>
-      <c r="G137" s="130"/>
+      <c r="B137" s="154"/>
+      <c r="C137" s="154"/>
+      <c r="D137" s="154"/>
+      <c r="E137" s="154"/>
+      <c r="F137" s="154"/>
+      <c r="G137" s="154"/>
     </row>
     <row r="138" spans="1:7" ht="60" customHeight="1">
-      <c r="A138" s="131" t="s">
+      <c r="A138" s="99" t="s">
         <v>130</v>
       </c>
-      <c r="B138" s="131"/>
-      <c r="C138" s="131"/>
-      <c r="D138" s="131"/>
-      <c r="E138" s="125" t="s">
+      <c r="B138" s="99"/>
+      <c r="C138" s="99"/>
+      <c r="D138" s="99"/>
+      <c r="E138" s="161" t="s">
         <v>103</v>
       </c>
-      <c r="F138" s="125"/>
-      <c r="G138" s="125"/>
+      <c r="F138" s="161"/>
+      <c r="G138" s="161"/>
     </row>
     <row r="139" spans="1:7" ht="54.75" customHeight="1">
-      <c r="A139" s="114" t="str">
+      <c r="A139" s="169" t="str">
         <f>G127</f>
         <v>-</v>
       </c>
-      <c r="B139" s="114"/>
-      <c r="C139" s="114"/>
-      <c r="D139" s="114"/>
-      <c r="E139" s="126" t="str">
+      <c r="B139" s="169"/>
+      <c r="C139" s="169"/>
+      <c r="D139" s="169"/>
+      <c r="E139" s="180" t="str">
         <f>VLOOKUP(A139,A133:G136,5,FALSE)</f>
         <v>-</v>
       </c>
-      <c r="F139" s="126"/>
-      <c r="G139" s="126"/>
+      <c r="F139" s="180"/>
+      <c r="G139" s="180"/>
     </row>
     <row r="142" spans="1:7" ht="15.75" thickBot="1"/>
     <row r="143" spans="1:7" ht="24" customHeight="1" thickBot="1">
-      <c r="A143" s="78" t="s">
+      <c r="A143" s="187" t="s">
         <v>141</v>
       </c>
-      <c r="B143" s="79"/>
-      <c r="C143" s="79"/>
-      <c r="D143" s="79"/>
-      <c r="E143" s="80">
+      <c r="B143" s="188"/>
+      <c r="C143" s="188"/>
+      <c r="D143" s="188"/>
+      <c r="E143" s="189">
         <f>E4</f>
         <v>0</v>
       </c>
-      <c r="F143" s="80"/>
-      <c r="G143" s="81"/>
+      <c r="F143" s="189"/>
+      <c r="G143" s="190"/>
     </row>
     <row r="144" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A144" s="115" t="s">
+      <c r="A144" s="170" t="s">
         <v>135</v>
       </c>
-      <c r="B144" s="116"/>
-      <c r="C144" s="116"/>
-      <c r="D144" s="116"/>
-      <c r="E144" s="116"/>
-      <c r="F144" s="116"/>
-      <c r="G144" s="117"/>
+      <c r="B144" s="171"/>
+      <c r="C144" s="171"/>
+      <c r="D144" s="171"/>
+      <c r="E144" s="171"/>
+      <c r="F144" s="171"/>
+      <c r="G144" s="172"/>
     </row>
     <row r="145" spans="1:7" ht="37.5" customHeight="1" thickBot="1">
-      <c r="A145" s="118" t="s">
+      <c r="A145" s="173" t="s">
         <v>136</v>
       </c>
-      <c r="B145" s="119"/>
-      <c r="C145" s="119"/>
-      <c r="D145" s="119"/>
-      <c r="E145" s="120" t="s">
+      <c r="B145" s="174"/>
+      <c r="C145" s="174"/>
+      <c r="D145" s="174"/>
+      <c r="E145" s="175" t="s">
         <v>137</v>
       </c>
-      <c r="F145" s="120"/>
-      <c r="G145" s="121"/>
+      <c r="F145" s="175"/>
+      <c r="G145" s="176"/>
     </row>
     <row r="146" spans="1:7" ht="30.75" customHeight="1" thickBot="1">
-      <c r="A146" s="108">
+      <c r="A146" s="163">
         <f>G4</f>
         <v>0</v>
       </c>
-      <c r="B146" s="109"/>
-      <c r="C146" s="109"/>
-      <c r="D146" s="109"/>
-      <c r="E146" s="122">
+      <c r="B146" s="164"/>
+      <c r="C146" s="164"/>
+      <c r="D146" s="164"/>
+      <c r="E146" s="177">
         <f>G4</f>
         <v>0</v>
       </c>
-      <c r="F146" s="123"/>
-      <c r="G146" s="124"/>
+      <c r="F146" s="178"/>
+      <c r="G146" s="179"/>
     </row>
     <row r="147" spans="1:7" ht="14.25" customHeight="1">
       <c r="A147" s="66" t="s">
@@ -4039,62 +4042,174 @@
       <c r="B147" s="67"/>
       <c r="C147" s="67"/>
       <c r="D147" s="67"/>
-      <c r="E147" s="72" t="s">
+      <c r="E147" s="181" t="s">
         <v>144</v>
       </c>
-      <c r="F147" s="72"/>
-      <c r="G147" s="73"/>
+      <c r="F147" s="181"/>
+      <c r="G147" s="182"/>
     </row>
     <row r="148" spans="1:7" ht="14.25" customHeight="1">
       <c r="A148" s="68"/>
       <c r="B148" s="69"/>
       <c r="C148" s="69"/>
       <c r="D148" s="69"/>
-      <c r="E148" s="74"/>
-      <c r="F148" s="74"/>
-      <c r="G148" s="75"/>
+      <c r="E148" s="183"/>
+      <c r="F148" s="183"/>
+      <c r="G148" s="184"/>
     </row>
     <row r="149" spans="1:7" ht="14.25" customHeight="1">
       <c r="A149" s="68"/>
       <c r="B149" s="69"/>
       <c r="C149" s="69"/>
       <c r="D149" s="69"/>
-      <c r="E149" s="74"/>
-      <c r="F149" s="74"/>
-      <c r="G149" s="75"/>
+      <c r="E149" s="183"/>
+      <c r="F149" s="183"/>
+      <c r="G149" s="184"/>
     </row>
     <row r="150" spans="1:7" ht="14.25" customHeight="1">
       <c r="A150" s="68"/>
       <c r="B150" s="69"/>
       <c r="C150" s="69"/>
       <c r="D150" s="69"/>
-      <c r="E150" s="74"/>
-      <c r="F150" s="74"/>
-      <c r="G150" s="75"/>
+      <c r="E150" s="183"/>
+      <c r="F150" s="183"/>
+      <c r="G150" s="184"/>
     </row>
     <row r="151" spans="1:7" ht="15" customHeight="1" thickBot="1">
       <c r="A151" s="70"/>
       <c r="B151" s="71"/>
       <c r="C151" s="71"/>
       <c r="D151" s="71"/>
-      <c r="E151" s="76"/>
-      <c r="F151" s="76"/>
-      <c r="G151" s="77"/>
+      <c r="E151" s="185"/>
+      <c r="F151" s="185"/>
+      <c r="G151" s="186"/>
     </row>
   </sheetData>
   <mergeCells count="160">
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="A1:C3"/>
-    <mergeCell ref="D1:G3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E147:G151"/>
+    <mergeCell ref="A143:D143"/>
+    <mergeCell ref="E143:G143"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="A122:G122"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="A123:C123"/>
+    <mergeCell ref="A124:C126"/>
+    <mergeCell ref="A127:F127"/>
+    <mergeCell ref="E136:G136"/>
+    <mergeCell ref="A133:D133"/>
+    <mergeCell ref="E133:G133"/>
+    <mergeCell ref="A114:F114"/>
+    <mergeCell ref="A115:F115"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="A117:F117"/>
+    <mergeCell ref="A118:F118"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A107:F107"/>
+    <mergeCell ref="A108:F108"/>
+    <mergeCell ref="A146:D146"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="C73:F73"/>
+    <mergeCell ref="A139:D139"/>
+    <mergeCell ref="A144:G144"/>
+    <mergeCell ref="A145:D145"/>
+    <mergeCell ref="E145:G145"/>
+    <mergeCell ref="E146:G146"/>
+    <mergeCell ref="E138:G138"/>
+    <mergeCell ref="E139:G139"/>
+    <mergeCell ref="A131:G131"/>
+    <mergeCell ref="A132:D132"/>
+    <mergeCell ref="A134:D134"/>
+    <mergeCell ref="A135:D135"/>
+    <mergeCell ref="A136:D136"/>
+    <mergeCell ref="A137:G137"/>
+    <mergeCell ref="A138:D138"/>
+    <mergeCell ref="E132:G132"/>
+    <mergeCell ref="E134:G134"/>
+    <mergeCell ref="E135:G135"/>
+    <mergeCell ref="A100:G100"/>
+    <mergeCell ref="A113:F113"/>
+    <mergeCell ref="A112:G112"/>
+    <mergeCell ref="A102:F102"/>
+    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="A104:F104"/>
+    <mergeCell ref="A105:F105"/>
+    <mergeCell ref="A106:F106"/>
+    <mergeCell ref="E96:G96"/>
+    <mergeCell ref="E97:G97"/>
+    <mergeCell ref="A101:G101"/>
+    <mergeCell ref="A89:G89"/>
+    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A95:G95"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="E90:G90"/>
+    <mergeCell ref="E92:G92"/>
+    <mergeCell ref="E93:G93"/>
+    <mergeCell ref="E94:G94"/>
+    <mergeCell ref="E91:G91"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A83:E85"/>
+    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="C72:F72"/>
+    <mergeCell ref="C74:F74"/>
+    <mergeCell ref="C75:F75"/>
+    <mergeCell ref="C76:F76"/>
+    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="B66:F66"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C56:F56"/>
+    <mergeCell ref="C57:F57"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A43:C45"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
@@ -4119,130 +4234,18 @@
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="E13:G13"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A43:C45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="A67:F67"/>
-    <mergeCell ref="A68:F68"/>
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="A71:G71"/>
-    <mergeCell ref="A51:G51"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="B62:F62"/>
-    <mergeCell ref="B64:F64"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="B66:F66"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="C57:F57"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="F86:G86"/>
-    <mergeCell ref="A82:E82"/>
-    <mergeCell ref="A86:E86"/>
-    <mergeCell ref="A83:E85"/>
-    <mergeCell ref="A81:G81"/>
-    <mergeCell ref="C72:F72"/>
-    <mergeCell ref="C74:F74"/>
-    <mergeCell ref="C75:F75"/>
-    <mergeCell ref="C76:F76"/>
-    <mergeCell ref="A77:F77"/>
-    <mergeCell ref="A78:F78"/>
-    <mergeCell ref="A89:G89"/>
-    <mergeCell ref="A90:D90"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A93:D93"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A95:G95"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="E90:G90"/>
-    <mergeCell ref="E92:G92"/>
-    <mergeCell ref="E93:G93"/>
-    <mergeCell ref="E94:G94"/>
-    <mergeCell ref="E91:G91"/>
-    <mergeCell ref="A113:F113"/>
-    <mergeCell ref="A112:G112"/>
-    <mergeCell ref="A102:F102"/>
-    <mergeCell ref="A103:F103"/>
-    <mergeCell ref="A104:F104"/>
-    <mergeCell ref="A105:F105"/>
-    <mergeCell ref="A106:F106"/>
-    <mergeCell ref="E96:G96"/>
-    <mergeCell ref="E97:G97"/>
-    <mergeCell ref="A101:G101"/>
-    <mergeCell ref="A146:D146"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="C73:F73"/>
-    <mergeCell ref="A139:D139"/>
-    <mergeCell ref="A144:G144"/>
-    <mergeCell ref="A145:D145"/>
-    <mergeCell ref="E145:G145"/>
-    <mergeCell ref="E146:G146"/>
-    <mergeCell ref="E138:G138"/>
-    <mergeCell ref="E139:G139"/>
-    <mergeCell ref="A131:G131"/>
-    <mergeCell ref="A132:D132"/>
-    <mergeCell ref="A134:D134"/>
-    <mergeCell ref="A135:D135"/>
-    <mergeCell ref="A136:D136"/>
-    <mergeCell ref="A137:G137"/>
-    <mergeCell ref="A138:D138"/>
-    <mergeCell ref="E132:G132"/>
-    <mergeCell ref="E134:G134"/>
-    <mergeCell ref="E135:G135"/>
-    <mergeCell ref="A100:G100"/>
-    <mergeCell ref="E147:G151"/>
-    <mergeCell ref="A143:D143"/>
-    <mergeCell ref="E143:G143"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="A122:G122"/>
-    <mergeCell ref="E123:F123"/>
-    <mergeCell ref="E124:F124"/>
-    <mergeCell ref="E125:F125"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="A123:C123"/>
-    <mergeCell ref="A124:C126"/>
-    <mergeCell ref="A127:F127"/>
-    <mergeCell ref="E136:G136"/>
-    <mergeCell ref="A133:D133"/>
-    <mergeCell ref="E133:G133"/>
-    <mergeCell ref="A114:F114"/>
-    <mergeCell ref="A115:F115"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="A117:F117"/>
-    <mergeCell ref="A118:F118"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A107:F107"/>
-    <mergeCell ref="A108:F108"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="A1:C3"/>
+    <mergeCell ref="D1:G3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:G11"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A29">
@@ -4281,10 +4284,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="33">
-      <c r="A1" s="222" t="s">
+      <c r="A1" s="220" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="222"/>
+      <c r="B1" s="220"/>
     </row>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="25" t="s">
@@ -4366,10 +4369,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="33">
-      <c r="A1" s="222" t="s">
+      <c r="A1" s="220" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="222"/>
+      <c r="B1" s="220"/>
     </row>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="25" t="s">
@@ -4451,11 +4454,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33">
-      <c r="A1" s="229" t="s">
+      <c r="A1" s="227" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="229"/>
-      <c r="C1" s="229"/>
+      <c r="B1" s="227"/>
+      <c r="C1" s="227"/>
     </row>
     <row r="2" spans="1:3" ht="92.25" customHeight="1">
       <c r="A2" s="21" t="s">
@@ -4469,7 +4472,7 @@
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="94" t="str">
+      <c r="A3" s="200" t="str">
         <f>IF('Γ2 ΙΣΤΟΡΙΚΟ ΣΥΜΜΟΡΦΩΣΗΣ'!B8="-",'Δ2 ΑΡΧΙΚΗ ΑΞΙΟΛΟΓΗΣΗ'!A3:A5+'Γ1 ΑΠΟΤΕΛΕΣΜΑ ΕΛΕΓΧΟΥ'!B8,"-")</f>
         <v>-</v>
       </c>
@@ -4481,7 +4484,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="94"/>
+      <c r="A4" s="200"/>
       <c r="B4" s="19" t="s">
         <v>90</v>
       </c>
@@ -4490,7 +4493,7 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="94"/>
+      <c r="A5" s="200"/>
       <c r="B5" s="12" t="s">
         <v>91</v>
       </c>
@@ -4506,11 +4509,11 @@
       <c r="A7" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="237" t="str">
+      <c r="B7" s="235" t="str">
         <f>IF($A$3&lt;=19,$C$3,IF($A$3&lt;=39,$C$4,IF($A$3="-","-",C$5)))</f>
         <v>-</v>
       </c>
-      <c r="C7" s="238"/>
+      <c r="C7" s="236"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4534,11 +4537,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="238" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="240"/>
-      <c r="C1" s="240"/>
+      <c r="B1" s="238"/>
+      <c r="C1" s="238"/>
       <c r="D1" s="20"/>
     </row>
     <row r="2" spans="1:4" ht="92.25" customHeight="1">
@@ -4553,7 +4556,7 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="94">
+      <c r="A3" s="200">
         <f>IF('Γ2 ΙΣΤΟΡΙΚΟ ΣΥΜΜΟΡΦΩΣΗΣ'!B8&lt;&gt;"-",SUM('Β1 ΤΥΠΟΣ ΠΛΗΡΟΤΗΤΑΣ'!C10+'B2 ΡΥΘΜΟΣ ΑΝΑΠΤΥΞΗΣ ΠΥΡΚΑΓΙΑΣ'!D8,'B3 ΠΛΗΘΟΣ ΧΡΗΣΤΩΝ'!C8+'Β4 ΚΤΙΡΙΑΚΗ ΠΟΛΥΠΛΟΚΟΤΗΤΑ'!C7+'Β5 ΜΕΤΑΔΟΣΗ ΠΥΡΚΑΓΙΑΣ'!C7+'Γ1 ΑΠΟΤΕΛΕΣΜΑ ΕΛΕΓΧΟΥ'!B8+'Γ2 ΙΣΤΟΡΙΚΟ ΣΥΜΜΟΡΦΩΣΗΣ'!B8),"-")</f>
         <v>52</v>
       </c>
@@ -4565,7 +4568,7 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="94"/>
+      <c r="A4" s="200"/>
       <c r="B4" s="19" t="s">
         <v>87</v>
       </c>
@@ -4574,7 +4577,7 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="94"/>
+      <c r="A5" s="200"/>
       <c r="B5" s="12" t="s">
         <v>88</v>
       </c>
@@ -4590,11 +4593,11 @@
       <c r="A7" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="239" t="str">
+      <c r="B7" s="237" t="str">
         <f>IF(A3="-","-",IF($A$3&lt;=21,$C$3,IF($A$3&lt;=43,$C$4,$C$5)))</f>
         <v>Υψηλό</v>
       </c>
-      <c r="C7" s="239"/>
+      <c r="C7" s="237"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4620,82 +4623,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="214" t="s">
+      <c r="A1" s="212" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="214"/>
-      <c r="C1" s="214"/>
-      <c r="D1" s="214"/>
+      <c r="B1" s="212"/>
+      <c r="C1" s="212"/>
+      <c r="D1" s="212"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="97" t="s">
+      <c r="B2" s="156" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="99"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="158"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="215" t="s">
+      <c r="B3" s="213" t="s">
         <v>104</v>
       </c>
-      <c r="C3" s="216"/>
-      <c r="D3" s="217"/>
+      <c r="C3" s="214"/>
+      <c r="D3" s="215"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="218" t="s">
+      <c r="B4" s="216" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="219"/>
-      <c r="D4" s="220"/>
+      <c r="C4" s="217"/>
+      <c r="D4" s="218"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="215" t="s">
+      <c r="B5" s="213" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="216"/>
-      <c r="D5" s="217"/>
+      <c r="C5" s="214"/>
+      <c r="D5" s="215"/>
     </row>
     <row r="6" spans="1:4" ht="15.75">
-      <c r="A6" s="130" t="s">
+      <c r="A6" s="154" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="130"/>
-      <c r="C6" s="130"/>
-      <c r="D6" s="130"/>
+      <c r="B6" s="154"/>
+      <c r="C6" s="154"/>
+      <c r="D6" s="154"/>
     </row>
     <row r="7" spans="1:4" ht="54" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="208" t="s">
+      <c r="B7" s="206" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="209"/>
-      <c r="D7" s="210"/>
+      <c r="C7" s="207"/>
+      <c r="D7" s="208"/>
     </row>
     <row r="8" spans="1:4" ht="88.5" customHeight="1">
       <c r="A8" s="36" t="str">
         <f>IF('Δ3 ΤΕΛΙΚΟ ΕΠΙΠΕΔΟ ΧΩΡΙΣ ΙΣΤΟΡΙΚ'!A3&lt;&gt;"-",'Δ3 ΤΕΛΙΚΟ ΕΠΙΠΕΔΟ ΧΩΡΙΣ ΙΣΤΟΡΙΚ'!B7,'Δ3 ΤΕΛΙΚΟ ΕΠΙΠΕΔΟ ΜΕ ΙΣΤΟΡΙΚΟ'!B7)</f>
         <v>Υψηλό</v>
       </c>
-      <c r="B8" s="241" t="str">
+      <c r="B8" s="239" t="str">
         <f>IF(A8=A3,B3,IF(A8=A4,B4,B5))</f>
         <v>Κάθε 12 μήνες</v>
       </c>
-      <c r="C8" s="242"/>
-      <c r="D8" s="243"/>
+      <c r="C8" s="240"/>
+      <c r="D8" s="241"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="20" t="s">
@@ -4734,82 +4737,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="214" t="s">
+      <c r="A1" s="212" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="214"/>
-      <c r="C1" s="214"/>
-      <c r="D1" s="214"/>
+      <c r="B1" s="212"/>
+      <c r="C1" s="212"/>
+      <c r="D1" s="212"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="97" t="s">
+      <c r="B2" s="156" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="99"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="158"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="215" t="s">
+      <c r="B3" s="213" t="s">
         <v>132</v>
       </c>
-      <c r="C3" s="216"/>
-      <c r="D3" s="217"/>
+      <c r="C3" s="214"/>
+      <c r="D3" s="215"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="218" t="s">
+      <c r="B4" s="216" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="219"/>
-      <c r="D4" s="220"/>
+      <c r="C4" s="217"/>
+      <c r="D4" s="218"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="215" t="s">
+      <c r="B5" s="213" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="216"/>
-      <c r="D5" s="217"/>
+      <c r="C5" s="214"/>
+      <c r="D5" s="215"/>
     </row>
     <row r="6" spans="1:4" ht="15.75">
-      <c r="A6" s="130" t="s">
+      <c r="A6" s="154" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="130"/>
-      <c r="C6" s="130"/>
-      <c r="D6" s="130"/>
+      <c r="B6" s="154"/>
+      <c r="C6" s="154"/>
+      <c r="D6" s="154"/>
     </row>
     <row r="7" spans="1:4" ht="36">
       <c r="A7" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="208" t="s">
+      <c r="B7" s="206" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="209"/>
-      <c r="D7" s="210"/>
+      <c r="C7" s="207"/>
+      <c r="D7" s="208"/>
     </row>
     <row r="8" spans="1:4" ht="84" customHeight="1">
       <c r="A8" s="36" t="str">
         <f>'Δ2 ΑΡΧΙΚΗ ΑΞΙΟΛΟΓΗΣΗ'!B6</f>
         <v>Υψηλό</v>
       </c>
-      <c r="B8" s="211" t="str">
+      <c r="B8" s="209" t="str">
         <f>IF(A8=A3,B3,IF(A8=A4,B4,B5))</f>
         <v>Κάθε 12 μήνες</v>
       </c>
-      <c r="C8" s="212"/>
-      <c r="D8" s="213"/>
+      <c r="C8" s="210"/>
+      <c r="D8" s="211"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -4846,11 +4849,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
-      <c r="A1" s="222" t="s">
+      <c r="A1" s="220" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="222"/>
-      <c r="C1" s="222"/>
+      <c r="B1" s="220"/>
+      <c r="C1" s="220"/>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1">
       <c r="A2" s="7" t="s">
@@ -4930,19 +4933,19 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="18">
-      <c r="A9" s="125" t="s">
+      <c r="A9" s="161" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="125"/>
+      <c r="B9" s="161"/>
       <c r="C9" s="10" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="33.75">
-      <c r="A10" s="221" t="s">
+      <c r="A10" s="219" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="221"/>
+      <c r="B10" s="219"/>
       <c r="C10" s="9">
         <f>IF($A$10=$A$3,$C$3,IF($A$10=$A$4,$C$4,IF($A$10=$A$5,$C$5,IF($A$10=$A$6,$C$6,IF($A$10=$A$7,$C$7,$C$8)))))</f>
         <v>16</v>
@@ -4978,12 +4981,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="214" t="s">
+      <c r="A1" s="212" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="214"/>
-      <c r="C1" s="214"/>
-      <c r="D1" s="214"/>
+      <c r="B1" s="212"/>
+      <c r="C1" s="212"/>
+      <c r="D1" s="212"/>
     </row>
     <row r="2" spans="1:4" ht="66.75" customHeight="1">
       <c r="A2" s="7" t="s">
@@ -5056,21 +5059,21 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="33.75" customHeight="1">
-      <c r="A7" s="173" t="s">
+      <c r="A7" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="174"/>
-      <c r="C7" s="175"/>
+      <c r="B7" s="115"/>
+      <c r="C7" s="116"/>
       <c r="D7" s="10" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="33.75">
-      <c r="A8" s="223">
+      <c r="A8" s="221">
         <v>4</v>
       </c>
-      <c r="B8" s="224"/>
-      <c r="C8" s="225"/>
+      <c r="B8" s="222"/>
+      <c r="C8" s="223"/>
       <c r="D8" s="37">
         <f>IF(A8=A3,D3,IF(A8=A4,D4,IF(A8=A5,D5,D6)))</f>
         <v>12</v>
@@ -5106,33 +5109,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33">
-      <c r="A1" s="229" t="s">
+      <c r="A1" s="227" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="229"/>
-      <c r="C1" s="229"/>
-      <c r="D1" s="229"/>
-      <c r="E1" s="229"/>
-      <c r="F1" s="229"/>
-      <c r="G1" s="229"/>
+      <c r="B1" s="227"/>
+      <c r="C1" s="227"/>
+      <c r="D1" s="227"/>
+      <c r="E1" s="227"/>
+      <c r="F1" s="227"/>
+      <c r="G1" s="227"/>
     </row>
     <row r="2" spans="1:7" ht="51" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="157" t="s">
+      <c r="B2" s="117" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157" t="s">
+      <c r="C2" s="117"/>
+      <c r="D2" s="117" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="157"/>
-      <c r="F2" s="157"/>
-      <c r="G2" s="157"/>
+      <c r="E2" s="117"/>
+      <c r="F2" s="117"/>
+      <c r="G2" s="117"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="164">
+      <c r="A3" s="124">
         <f>SUM('Β1 ΤΥΠΟΣ ΠΛΗΡΟΤΗΤΑΣ'!C10+'B2 ΡΥΘΜΟΣ ΑΝΑΠΤΥΞΗΣ ΠΥΡΚΑΓΙΑΣ'!D8)</f>
         <v>28</v>
       </c>
@@ -5142,68 +5145,68 @@
       <c r="C3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="96" t="s">
+      <c r="D3" s="110" t="s">
         <v>124</v>
       </c>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="164"/>
+      <c r="A4" s="124"/>
       <c r="B4" s="12" t="s">
         <v>33</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="96" t="s">
+      <c r="D4" s="110" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="96"/>
-      <c r="F4" s="96"/>
-      <c r="G4" s="96"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="164"/>
+      <c r="A5" s="124"/>
       <c r="B5" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="96"/>
-      <c r="E5" s="96"/>
-      <c r="F5" s="96"/>
-      <c r="G5" s="96"/>
+      <c r="D5" s="110"/>
+      <c r="E5" s="110"/>
+      <c r="F5" s="110"/>
+      <c r="G5" s="110"/>
     </row>
     <row r="6" spans="1:7" ht="33.75">
-      <c r="A6" s="228" t="s">
+      <c r="A6" s="226" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="228"/>
+      <c r="B6" s="226"/>
       <c r="C6" s="9" t="str">
         <f>IF($A$3&lt;=8,$C$3,IF($A$3&lt;=18,$C$4,$C$5))</f>
         <v>Υψηλό</v>
       </c>
-      <c r="D6" s="221" t="str">
+      <c r="D6" s="219" t="str">
         <f>IF($A$3&lt;=8,$D$3,$D$4)</f>
         <v>ΝΑΙ</v>
       </c>
-      <c r="E6" s="221"/>
-      <c r="F6" s="221"/>
-      <c r="G6" s="221"/>
+      <c r="E6" s="219"/>
+      <c r="F6" s="219"/>
+      <c r="G6" s="219"/>
     </row>
     <row r="7" spans="1:7" ht="42" customHeight="1">
-      <c r="A7" s="226" t="s">
+      <c r="A7" s="224" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="227"/>
-      <c r="C7" s="227"/>
-      <c r="D7" s="227"/>
-      <c r="E7" s="227"/>
-      <c r="F7" s="227"/>
-      <c r="G7" s="227"/>
+      <c r="B7" s="225"/>
+      <c r="C7" s="225"/>
+      <c r="D7" s="225"/>
+      <c r="E7" s="225"/>
+      <c r="F7" s="225"/>
+      <c r="G7" s="225"/>
     </row>
     <row r="9" spans="1:7" ht="66.75" customHeight="1"/>
   </sheetData>
@@ -5235,11 +5238,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="34.5">
-      <c r="A1" s="230" t="s">
+      <c r="A1" s="228" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="230"/>
-      <c r="C1" s="230"/>
+      <c r="B1" s="228"/>
+      <c r="C1" s="228"/>
     </row>
     <row r="2" spans="1:3" ht="15.75">
       <c r="A2" s="15" t="s">
@@ -5297,19 +5300,19 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="60.75" customHeight="1">
-      <c r="A7" s="131" t="s">
+      <c r="A7" s="99" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="131"/>
+      <c r="B7" s="99"/>
       <c r="C7" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="33.75">
-      <c r="A8" s="221" t="s">
+      <c r="A8" s="219" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="221"/>
+      <c r="B8" s="219"/>
       <c r="C8" s="9">
         <f>IF($A$8=$A$3,$C$3,IF($A$8=$A$4,$C$4,IF($A$8=$A$5,$C$5,$C$6)))</f>
         <v>6</v>
@@ -5343,11 +5346,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33">
-      <c r="A1" s="222" t="s">
+      <c r="A1" s="220" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="222"/>
-      <c r="C1" s="222"/>
+      <c r="B1" s="220"/>
+      <c r="C1" s="220"/>
     </row>
     <row r="2" spans="1:3" ht="15.75">
       <c r="A2" s="15" t="s">
@@ -5394,19 +5397,19 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" customHeight="1">
-      <c r="A6" s="231" t="s">
+      <c r="A6" s="229" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="231"/>
+      <c r="B6" s="229"/>
       <c r="C6" s="17" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="33.75">
-      <c r="A7" s="221" t="s">
+      <c r="A7" s="219" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="221"/>
+      <c r="B7" s="219"/>
       <c r="C7" s="9">
         <f>IF($A$7=$A$3,$C$3,IF($A$7=$A$4,$C$4,$C$5))</f>
         <v>0</v>
@@ -5441,12 +5444,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33">
-      <c r="A1" s="222" t="s">
+      <c r="A1" s="220" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="222"/>
-      <c r="C1" s="222"/>
-      <c r="D1" s="222"/>
+      <c r="B1" s="220"/>
+      <c r="C1" s="220"/>
+      <c r="D1" s="220"/>
     </row>
     <row r="2" spans="1:4" ht="15.75">
       <c r="A2" s="15" t="s">
@@ -5505,25 +5508,25 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="51.75" customHeight="1">
-      <c r="A6" s="150" t="s">
+      <c r="A6" s="151" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="150"/>
-      <c r="C6" s="232" t="s">
+      <c r="B6" s="151"/>
+      <c r="C6" s="230" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="233"/>
+      <c r="D6" s="231"/>
     </row>
     <row r="7" spans="1:4" ht="33.75">
-      <c r="A7" s="221">
+      <c r="A7" s="219">
         <v>1</v>
       </c>
-      <c r="B7" s="221"/>
-      <c r="C7" s="223">
+      <c r="B7" s="219"/>
+      <c r="C7" s="221">
         <f>IF($A$7=$A$3,$D$3,IF($A$7=$A$4,$D$4,$D$5))</f>
         <v>0</v>
       </c>
-      <c r="D7" s="225"/>
+      <c r="D7" s="223"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5555,11 +5558,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33">
-      <c r="A1" s="234" t="s">
+      <c r="A1" s="232" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="234"/>
-      <c r="C1" s="234"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="232"/>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
       <c r="F1" s="18"/>
@@ -5569,13 +5572,13 @@
       <c r="A2" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="235" t="s">
+      <c r="B2" s="233" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="235"/>
+      <c r="C2" s="233"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="236">
+      <c r="A3" s="234">
         <f>SUM('Β1 ΤΥΠΟΣ ΠΛΗΡΟΤΗΤΑΣ'!C10+'B2 ΡΥΘΜΟΣ ΑΝΑΠΤΥΞΗΣ ΠΥΡΚΑΓΙΑΣ'!D8,'B3 ΠΛΗΘΟΣ ΧΡΗΣΤΩΝ'!C8+'Β4 ΚΤΙΡΙΑΚΗ ΠΟΛΥΠΛΟΚΟΤΗΤΑ'!C7+'Β5 ΜΕΤΑΔΟΣΗ ΠΥΡΚΑΓΙΑΣ'!C7)</f>
         <v>34</v>
       </c>
@@ -5587,7 +5590,7 @@
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="236"/>
+      <c r="A4" s="234"/>
       <c r="B4" s="19" t="s">
         <v>69</v>
       </c>
@@ -5596,7 +5599,7 @@
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="236"/>
+      <c r="A5" s="234"/>
       <c r="B5" s="12" t="s">
         <v>70</v>
       </c>
@@ -5608,11 +5611,11 @@
       <c r="A6" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="223" t="str">
+      <c r="B6" s="221" t="str">
         <f>IF($A$3&lt;=14,$C$3,IF($A$3&lt;=30,$C$4,C$5))</f>
         <v>Υψηλό</v>
       </c>
-      <c r="C6" s="225"/>
+      <c r="C6" s="223"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
change exceljs to xlsxpopulate package
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -23,6 +23,13 @@
     <sheet name="Συχνότητα Ελέγχων Τελικής Αξιολ" sheetId="13" r:id="rId14"/>
   </sheets>
   <definedNames>
+    <definedName name="APOT_ELEG">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$103:$F$106</definedName>
+    <definedName name="APOTELEG">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$103:$F$106</definedName>
+    <definedName name="ASS">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$103:$A$106</definedName>
+    <definedName name="ISTORIKO_SYM">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$114:$A$117</definedName>
+    <definedName name="ktiriaki_pol">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$63:$A$66</definedName>
+    <definedName name="metadosi">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$73:$A$76</definedName>
+    <definedName name="PLITHOS">'ΣΤΟΙΧΕΙΑ ΕΠΙΧΕΙΡΗΣΗΣ'!$A$53:$A$57</definedName>
     <definedName name="Table1">#REF!</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
@@ -43,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="145">
   <si>
     <t>Τύπος Πληρότητας</t>
   </si>
@@ -530,9 +537,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
-  </numFmts>
   <fonts count="35">
     <font>
       <sz val="11"/>
@@ -893,7 +897,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -1222,36 +1226,6 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom style="medium">
         <color indexed="64"/>
@@ -1263,7 +1237,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="244">
+  <cellXfs count="254">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1478,103 +1452,110 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -1588,6 +1569,32 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="10" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1691,77 +1698,178 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="24" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1771,18 +1879,6 @@
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1822,90 +1918,6 @@
     <xf numFmtId="0" fontId="31" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2013,14 +2025,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2423,73 +2427,74 @@
     <col min="4" max="4" width="21.42578125" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="26.5703125" customWidth="1"/>
+    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A1" s="74"/>
-      <c r="B1" s="75"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="80" t="s">
+      <c r="A1" s="83"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="89" t="s">
         <v>109</v>
       </c>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A2" s="77"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
+      <c r="A2" s="86"/>
+      <c r="B2" s="87"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
     </row>
     <row r="3" spans="1:7" ht="19.149999999999999" customHeight="1" thickBot="1">
-      <c r="A3" s="77"/>
-      <c r="B3" s="78"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
+      <c r="A3" s="86"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="82" t="s">
+      <c r="A4" s="91" t="s">
         <v>110</v>
       </c>
-      <c r="B4" s="83"/>
-      <c r="C4" s="84"/>
-      <c r="D4" s="93" t="s">
+      <c r="B4" s="92"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="108" t="s">
         <v>111</v>
       </c>
-      <c r="E4" s="95"/>
-      <c r="F4" s="191" t="s">
+      <c r="E4" s="103"/>
+      <c r="F4" s="172" t="s">
         <v>112</v>
       </c>
-      <c r="G4" s="242"/>
+      <c r="G4" s="174"/>
     </row>
     <row r="5" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A5" s="85" t="s">
+      <c r="A5" s="94" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="86"/>
-      <c r="C5" s="87"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="96"/>
-      <c r="F5" s="192"/>
-      <c r="G5" s="243"/>
+      <c r="B5" s="95"/>
+      <c r="C5" s="96"/>
+      <c r="D5" s="109"/>
+      <c r="E5" s="104"/>
+      <c r="F5" s="173"/>
+      <c r="G5" s="175"/>
     </row>
     <row r="6" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A6" s="100" t="s">
+      <c r="A6" s="114" t="s">
         <v>142</v>
       </c>
-      <c r="B6" s="101"/>
-      <c r="C6" s="101"/>
-      <c r="D6" s="102"/>
-      <c r="E6" s="103"/>
-      <c r="F6" s="103"/>
-      <c r="G6" s="104"/>
+      <c r="B6" s="115"/>
+      <c r="C6" s="115"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="106"/>
+      <c r="G6" s="107"/>
     </row>
     <row r="7" spans="1:7" ht="15.75" thickBot="1"/>
     <row r="8" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
@@ -2504,127 +2509,127 @@
       <c r="G8" s="45"/>
     </row>
     <row r="9" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A9" s="88" t="s">
+      <c r="A9" s="97" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="88"/>
-      <c r="C9" s="88"/>
-      <c r="D9" s="88"/>
-      <c r="E9" s="89"/>
-      <c r="F9" s="89"/>
-      <c r="G9" s="89"/>
+      <c r="B9" s="97"/>
+      <c r="C9" s="97"/>
+      <c r="D9" s="97"/>
+      <c r="E9" s="98"/>
+      <c r="F9" s="98"/>
+      <c r="G9" s="98"/>
     </row>
     <row r="10" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A10" s="72" t="s">
+      <c r="A10" s="99" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="72"/>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="89"/>
+      <c r="B10" s="99"/>
+      <c r="C10" s="99"/>
+      <c r="D10" s="99"/>
+      <c r="E10" s="98"/>
+      <c r="F10" s="98"/>
+      <c r="G10" s="98"/>
     </row>
     <row r="11" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A11" s="88" t="s">
+      <c r="A11" s="97" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="88"/>
-      <c r="C11" s="88"/>
-      <c r="D11" s="88"/>
-      <c r="E11" s="90"/>
-      <c r="F11" s="91"/>
-      <c r="G11" s="92"/>
+      <c r="B11" s="97"/>
+      <c r="C11" s="97"/>
+      <c r="D11" s="97"/>
+      <c r="E11" s="100"/>
+      <c r="F11" s="101"/>
+      <c r="G11" s="102"/>
     </row>
     <row r="12" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A12" s="72" t="s">
+      <c r="A12" s="99" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="72"/>
-      <c r="C12" s="72"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
-      <c r="G12" s="73"/>
+      <c r="B12" s="99"/>
+      <c r="C12" s="99"/>
+      <c r="D12" s="99"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
     </row>
     <row r="13" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="97" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="88"/>
-      <c r="C13" s="88"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="91"/>
-      <c r="G13" s="92"/>
+      <c r="B13" s="97"/>
+      <c r="C13" s="97"/>
+      <c r="D13" s="97"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="101"/>
+      <c r="G13" s="102"/>
     </row>
     <row r="14" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A14" s="72" t="s">
+      <c r="A14" s="99" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="72"/>
-      <c r="C14" s="72"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="73"/>
-      <c r="F14" s="73"/>
-      <c r="G14" s="73"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="110"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="110"/>
     </row>
     <row r="15" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A15" s="88" t="s">
+      <c r="A15" s="97" t="s">
         <v>121</v>
       </c>
-      <c r="B15" s="88"/>
-      <c r="C15" s="88"/>
-      <c r="D15" s="88"/>
-      <c r="E15" s="89"/>
-      <c r="F15" s="89"/>
-      <c r="G15" s="89"/>
+      <c r="B15" s="97"/>
+      <c r="C15" s="97"/>
+      <c r="D15" s="97"/>
+      <c r="E15" s="98"/>
+      <c r="F15" s="98"/>
+      <c r="G15" s="98"/>
     </row>
     <row r="16" spans="1:7" ht="49.9" customHeight="1" thickBot="1">
-      <c r="A16" s="72" t="s">
+      <c r="A16" s="99" t="s">
         <v>122</v>
       </c>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="73"/>
-      <c r="F16" s="73"/>
-      <c r="G16" s="73"/>
+      <c r="B16" s="99"/>
+      <c r="C16" s="99"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="110"/>
+      <c r="F16" s="110"/>
+      <c r="G16" s="110"/>
     </row>
     <row r="17" spans="1:7" ht="49.5" customHeight="1" thickBot="1">
-      <c r="A17" s="88" t="s">
+      <c r="A17" s="97" t="s">
         <v>123</v>
       </c>
-      <c r="B17" s="88"/>
-      <c r="C17" s="88"/>
-      <c r="D17" s="88"/>
-      <c r="E17" s="105"/>
-      <c r="F17" s="89"/>
-      <c r="G17" s="89"/>
+      <c r="B17" s="97"/>
+      <c r="C17" s="97"/>
+      <c r="D17" s="97"/>
+      <c r="E17" s="116"/>
+      <c r="F17" s="98"/>
+      <c r="G17" s="98"/>
     </row>
     <row r="19" spans="1:7" hidden="1"/>
     <row r="20" spans="1:7" ht="26.25">
-      <c r="A20" s="106" t="s">
+      <c r="A20" s="117" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="106"/>
-      <c r="C20" s="106"/>
-      <c r="D20" s="106"/>
-      <c r="E20" s="106"/>
-      <c r="F20" s="106"/>
-      <c r="G20" s="106"/>
+      <c r="B20" s="117"/>
+      <c r="C20" s="117"/>
+      <c r="D20" s="117"/>
+      <c r="E20" s="117"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
     </row>
     <row r="21" spans="1:7" ht="63">
       <c r="A21" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="107" t="s">
+      <c r="B21" s="118" t="s">
         <v>2</v>
       </c>
-      <c r="C21" s="108"/>
-      <c r="D21" s="108"/>
-      <c r="E21" s="108"/>
-      <c r="F21" s="109"/>
+      <c r="C21" s="119"/>
+      <c r="D21" s="119"/>
+      <c r="E21" s="119"/>
+      <c r="F21" s="120"/>
       <c r="G21" s="47" t="s">
         <v>3</v>
       </c>
@@ -2633,13 +2638,13 @@
       <c r="A22" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="110" t="s">
+      <c r="B22" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="110"/>
-      <c r="D22" s="110"/>
-      <c r="E22" s="110"/>
-      <c r="F22" s="110"/>
+      <c r="C22" s="121"/>
+      <c r="D22" s="121"/>
+      <c r="E22" s="121"/>
+      <c r="F22" s="121"/>
       <c r="G22" s="42">
         <v>0</v>
       </c>
@@ -2648,13 +2653,13 @@
       <c r="A23" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="111" t="s">
+      <c r="B23" s="122" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="111"/>
-      <c r="D23" s="111"/>
-      <c r="E23" s="111"/>
-      <c r="F23" s="111"/>
+      <c r="C23" s="122"/>
+      <c r="D23" s="122"/>
+      <c r="E23" s="122"/>
+      <c r="F23" s="122"/>
       <c r="G23" s="5">
         <v>8</v>
       </c>
@@ -2663,13 +2668,13 @@
       <c r="A24" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="110" t="s">
+      <c r="B24" s="121" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="110"/>
-      <c r="D24" s="110"/>
-      <c r="E24" s="110"/>
-      <c r="F24" s="110"/>
+      <c r="C24" s="121"/>
+      <c r="D24" s="121"/>
+      <c r="E24" s="121"/>
+      <c r="F24" s="121"/>
       <c r="G24" s="42">
         <v>4</v>
       </c>
@@ -2678,13 +2683,13 @@
       <c r="A25" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="111" t="s">
+      <c r="B25" s="122" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="111"/>
-      <c r="D25" s="111"/>
-      <c r="E25" s="111"/>
-      <c r="F25" s="111"/>
+      <c r="C25" s="122"/>
+      <c r="D25" s="122"/>
+      <c r="E25" s="122"/>
+      <c r="F25" s="122"/>
       <c r="G25" s="5">
         <v>12</v>
       </c>
@@ -2693,13 +2698,13 @@
       <c r="A26" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="112" t="s">
+      <c r="B26" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="112"/>
-      <c r="D26" s="112"/>
-      <c r="E26" s="112"/>
-      <c r="F26" s="112"/>
+      <c r="C26" s="123"/>
+      <c r="D26" s="123"/>
+      <c r="E26" s="123"/>
+      <c r="F26" s="123"/>
       <c r="G26" s="42">
         <v>12</v>
       </c>
@@ -2708,54 +2713,54 @@
       <c r="A27" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="97" t="s">
+      <c r="B27" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="97"/>
-      <c r="D27" s="97"/>
-      <c r="E27" s="97"/>
-      <c r="F27" s="97"/>
+      <c r="C27" s="111"/>
+      <c r="D27" s="111"/>
+      <c r="E27" s="111"/>
+      <c r="F27" s="111"/>
       <c r="G27" s="5">
         <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="38.25" customHeight="1">
-      <c r="A28" s="114" t="s">
+      <c r="A28" s="125" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="115"/>
-      <c r="C28" s="115"/>
-      <c r="D28" s="115"/>
-      <c r="E28" s="115"/>
-      <c r="F28" s="116"/>
+      <c r="B28" s="126"/>
+      <c r="C28" s="126"/>
+      <c r="D28" s="126"/>
+      <c r="E28" s="126"/>
+      <c r="F28" s="127"/>
       <c r="G28" s="41" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A29" s="98" t="s">
+      <c r="A29" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="98"/>
-      <c r="C29" s="98"/>
-      <c r="D29" s="98"/>
-      <c r="E29" s="98"/>
-      <c r="F29" s="98"/>
+      <c r="B29" s="112"/>
+      <c r="C29" s="112"/>
+      <c r="D29" s="112"/>
+      <c r="E29" s="112"/>
+      <c r="F29" s="112"/>
       <c r="G29" s="55">
         <f>VLOOKUP(A29,A22:G27,7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="26.25">
-      <c r="A31" s="106" t="s">
+      <c r="A31" s="117" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="106"/>
-      <c r="C31" s="106"/>
-      <c r="D31" s="106"/>
-      <c r="E31" s="106"/>
-      <c r="F31" s="106"/>
-      <c r="G31" s="106"/>
+      <c r="B31" s="117"/>
+      <c r="C31" s="117"/>
+      <c r="D31" s="117"/>
+      <c r="E31" s="117"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="117"/>
     </row>
     <row r="32" spans="1:7" ht="45">
       <c r="A32" s="51" t="s">
@@ -2764,12 +2769,12 @@
       <c r="B32" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="C32" s="107" t="s">
+      <c r="C32" s="118" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="108"/>
-      <c r="E32" s="108"/>
-      <c r="F32" s="109"/>
+      <c r="D32" s="119"/>
+      <c r="E32" s="119"/>
+      <c r="F32" s="120"/>
       <c r="G32" s="49" t="s">
         <v>3</v>
       </c>
@@ -2781,12 +2786,12 @@
       <c r="B33" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="112" t="s">
+      <c r="C33" s="123" t="s">
         <v>22</v>
       </c>
-      <c r="D33" s="112"/>
-      <c r="E33" s="112"/>
-      <c r="F33" s="112"/>
+      <c r="D33" s="123"/>
+      <c r="E33" s="123"/>
+      <c r="F33" s="123"/>
       <c r="G33" s="42">
         <v>0</v>
       </c>
@@ -2798,12 +2803,12 @@
       <c r="B34" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="97" t="s">
+      <c r="C34" s="111" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="97"/>
-      <c r="E34" s="97"/>
-      <c r="F34" s="97"/>
+      <c r="D34" s="111"/>
+      <c r="E34" s="111"/>
+      <c r="F34" s="111"/>
       <c r="G34" s="5">
         <v>4</v>
       </c>
@@ -2815,12 +2820,12 @@
       <c r="B35" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="112" t="s">
+      <c r="C35" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="112"/>
-      <c r="E35" s="112"/>
-      <c r="F35" s="112"/>
+      <c r="D35" s="123"/>
+      <c r="E35" s="123"/>
+      <c r="F35" s="123"/>
       <c r="G35" s="42">
         <v>8</v>
       </c>
@@ -2832,142 +2837,142 @@
       <c r="B36" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="97" t="s">
+      <c r="C36" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="97"/>
-      <c r="E36" s="97"/>
-      <c r="F36" s="97"/>
+      <c r="D36" s="111"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="111"/>
       <c r="G36" s="5">
         <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="42.75" customHeight="1">
-      <c r="A37" s="99" t="s">
+      <c r="A37" s="113" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="99"/>
-      <c r="C37" s="99"/>
-      <c r="D37" s="99"/>
-      <c r="E37" s="99"/>
-      <c r="F37" s="99"/>
+      <c r="B37" s="113"/>
+      <c r="C37" s="113"/>
+      <c r="D37" s="113"/>
+      <c r="E37" s="113"/>
+      <c r="F37" s="113"/>
       <c r="G37" s="41" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A38" s="98">
+      <c r="A38" s="112">
         <v>1</v>
       </c>
-      <c r="B38" s="98"/>
-      <c r="C38" s="98"/>
-      <c r="D38" s="98"/>
-      <c r="E38" s="98"/>
-      <c r="F38" s="98"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
       <c r="G38" s="55">
         <f>VLOOKUP(A38,A33:G36,7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="30">
-      <c r="A41" s="113" t="s">
+      <c r="A41" s="124" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="113"/>
-      <c r="C41" s="113"/>
-      <c r="D41" s="113"/>
-      <c r="E41" s="113"/>
-      <c r="F41" s="113"/>
-      <c r="G41" s="113"/>
+      <c r="B41" s="124"/>
+      <c r="C41" s="124"/>
+      <c r="D41" s="124"/>
+      <c r="E41" s="124"/>
+      <c r="F41" s="124"/>
+      <c r="G41" s="124"/>
     </row>
     <row r="42" spans="1:7" ht="30">
-      <c r="A42" s="123" t="s">
+      <c r="A42" s="134" t="s">
         <v>28</v>
       </c>
-      <c r="B42" s="123"/>
-      <c r="C42" s="123"/>
-      <c r="D42" s="117" t="s">
+      <c r="B42" s="134"/>
+      <c r="C42" s="134"/>
+      <c r="D42" s="128" t="s">
         <v>29</v>
       </c>
-      <c r="E42" s="117"/>
-      <c r="F42" s="117"/>
+      <c r="E42" s="128"/>
+      <c r="F42" s="128"/>
       <c r="G42" s="48" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15" customHeight="1">
-      <c r="A43" s="124">
+      <c r="A43" s="135">
         <f>SUM(G29,G38)</f>
         <v>0</v>
       </c>
-      <c r="B43" s="124"/>
-      <c r="C43" s="124"/>
+      <c r="B43" s="135"/>
+      <c r="C43" s="135"/>
       <c r="D43" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E43" s="128" t="s">
+      <c r="E43" s="139" t="s">
         <v>34</v>
       </c>
-      <c r="F43" s="128"/>
+      <c r="F43" s="139"/>
       <c r="G43" s="42" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15" customHeight="1">
-      <c r="A44" s="124"/>
-      <c r="B44" s="124"/>
-      <c r="C44" s="124"/>
+      <c r="A44" s="135"/>
+      <c r="B44" s="135"/>
+      <c r="C44" s="135"/>
       <c r="D44" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E44" s="128" t="s">
+      <c r="E44" s="139" t="s">
         <v>35</v>
       </c>
-      <c r="F44" s="128"/>
-      <c r="G44" s="125" t="s">
+      <c r="F44" s="139"/>
+      <c r="G44" s="136" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15" customHeight="1">
-      <c r="A45" s="124"/>
-      <c r="B45" s="124"/>
-      <c r="C45" s="124"/>
+      <c r="A45" s="135"/>
+      <c r="B45" s="135"/>
+      <c r="C45" s="135"/>
       <c r="D45" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E45" s="128" t="s">
+      <c r="E45" s="139" t="s">
         <v>36</v>
       </c>
-      <c r="F45" s="128"/>
-      <c r="G45" s="126"/>
+      <c r="F45" s="139"/>
+      <c r="G45" s="137"/>
     </row>
     <row r="46" spans="1:7" ht="44.25" customHeight="1">
-      <c r="A46" s="120" t="s">
+      <c r="A46" s="131" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="121"/>
-      <c r="C46" s="121"/>
-      <c r="D46" s="122"/>
-      <c r="E46" s="118" t="str">
+      <c r="B46" s="132"/>
+      <c r="C46" s="132"/>
+      <c r="D46" s="133"/>
+      <c r="E46" s="129" t="str">
         <f>IF(A43&lt;=8,E43,IF(AND(A43&gt;=9,A43&lt;=18),E44,E45))</f>
         <v>Χαμηλό</v>
       </c>
-      <c r="F46" s="119"/>
+      <c r="F46" s="130"/>
       <c r="G46" s="57" t="str">
         <f>IF(A43&gt;8,G44,G43)</f>
         <v>ΌΧΙ*</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="41.25" customHeight="1">
-      <c r="A47" s="127" t="s">
+      <c r="A47" s="138" t="s">
         <v>125</v>
       </c>
-      <c r="B47" s="127"/>
-      <c r="C47" s="127"/>
-      <c r="D47" s="127"/>
-      <c r="E47" s="127"/>
-      <c r="F47" s="127"/>
-      <c r="G47" s="127"/>
+      <c r="B47" s="138"/>
+      <c r="C47" s="138"/>
+      <c r="D47" s="138"/>
+      <c r="E47" s="138"/>
+      <c r="F47" s="138"/>
+      <c r="G47" s="138"/>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="44"/>
@@ -2979,167 +2984,167 @@
       <c r="G48" s="44"/>
     </row>
     <row r="50" spans="1:7" ht="24">
-      <c r="A50" s="165" t="s">
+      <c r="A50" s="189" t="s">
         <v>138</v>
       </c>
-      <c r="B50" s="165"/>
-      <c r="C50" s="165"/>
-      <c r="D50" s="165"/>
-      <c r="E50" s="165"/>
-      <c r="F50" s="165"/>
-      <c r="G50" s="165"/>
+      <c r="B50" s="189"/>
+      <c r="C50" s="189"/>
+      <c r="D50" s="189"/>
+      <c r="E50" s="189"/>
+      <c r="F50" s="189"/>
+      <c r="G50" s="189"/>
     </row>
     <row r="51" spans="1:7" ht="26.25">
-      <c r="A51" s="106" t="s">
+      <c r="A51" s="117" t="s">
         <v>40</v>
       </c>
-      <c r="B51" s="106"/>
-      <c r="C51" s="106"/>
-      <c r="D51" s="106"/>
-      <c r="E51" s="106"/>
-      <c r="F51" s="106"/>
-      <c r="G51" s="106"/>
+      <c r="B51" s="117"/>
+      <c r="C51" s="117"/>
+      <c r="D51" s="117"/>
+      <c r="E51" s="117"/>
+      <c r="F51" s="117"/>
+      <c r="G51" s="117"/>
     </row>
     <row r="52" spans="1:7" ht="15.75">
-      <c r="A52" s="138" t="s">
+      <c r="A52" s="149" t="s">
         <v>41</v>
       </c>
-      <c r="B52" s="138"/>
-      <c r="C52" s="138" t="s">
+      <c r="B52" s="149"/>
+      <c r="C52" s="149" t="s">
         <v>45</v>
       </c>
-      <c r="D52" s="138"/>
-      <c r="E52" s="138"/>
-      <c r="F52" s="138"/>
+      <c r="D52" s="149"/>
+      <c r="E52" s="149"/>
+      <c r="F52" s="149"/>
       <c r="G52" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:7">
-      <c r="A53" s="110" t="s">
+      <c r="A53" s="75" t="s">
         <v>126</v>
       </c>
-      <c r="B53" s="110"/>
-      <c r="C53" s="110" t="s">
+      <c r="B53" s="77"/>
+      <c r="C53" s="121" t="s">
         <v>126</v>
       </c>
-      <c r="D53" s="110"/>
-      <c r="E53" s="110"/>
-      <c r="F53" s="110"/>
+      <c r="D53" s="121"/>
+      <c r="E53" s="121"/>
+      <c r="F53" s="121"/>
       <c r="G53" s="42" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="54" spans="1:7">
-      <c r="A54" s="110" t="s">
+      <c r="A54" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="B54" s="110"/>
-      <c r="C54" s="110" t="s">
+      <c r="B54" s="77"/>
+      <c r="C54" s="121" t="s">
         <v>46</v>
       </c>
-      <c r="D54" s="110"/>
-      <c r="E54" s="110"/>
-      <c r="F54" s="110"/>
+      <c r="D54" s="121"/>
+      <c r="E54" s="121"/>
+      <c r="F54" s="121"/>
       <c r="G54" s="42">
         <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:7">
-      <c r="A55" s="137" t="s">
+      <c r="A55" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="B55" s="137"/>
-      <c r="C55" s="137" t="s">
+      <c r="B55" s="82"/>
+      <c r="C55" s="148" t="s">
         <v>47</v>
       </c>
-      <c r="D55" s="137"/>
-      <c r="E55" s="137"/>
-      <c r="F55" s="137"/>
+      <c r="D55" s="148"/>
+      <c r="E55" s="148"/>
+      <c r="F55" s="148"/>
       <c r="G55" s="13">
         <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:7">
-      <c r="A56" s="110" t="s">
+      <c r="A56" s="75" t="s">
         <v>43</v>
       </c>
-      <c r="B56" s="110"/>
-      <c r="C56" s="110" t="s">
+      <c r="B56" s="77"/>
+      <c r="C56" s="121" t="s">
         <v>48</v>
       </c>
-      <c r="D56" s="110"/>
-      <c r="E56" s="110"/>
-      <c r="F56" s="110"/>
+      <c r="D56" s="121"/>
+      <c r="E56" s="121"/>
+      <c r="F56" s="121"/>
       <c r="G56" s="42">
         <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:7">
-      <c r="A57" s="137" t="s">
+      <c r="A57" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="B57" s="137"/>
-      <c r="C57" s="137" t="s">
+      <c r="B57" s="82"/>
+      <c r="C57" s="148" t="s">
         <v>49</v>
       </c>
-      <c r="D57" s="137"/>
-      <c r="E57" s="137"/>
-      <c r="F57" s="137"/>
+      <c r="D57" s="148"/>
+      <c r="E57" s="148"/>
+      <c r="F57" s="148"/>
       <c r="G57" s="13">
         <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="18" customHeight="1">
-      <c r="A58" s="99" t="s">
+      <c r="A58" s="113" t="s">
         <v>64</v>
       </c>
-      <c r="B58" s="99"/>
-      <c r="C58" s="99"/>
-      <c r="D58" s="99"/>
-      <c r="E58" s="99"/>
-      <c r="F58" s="99"/>
+      <c r="B58" s="113"/>
+      <c r="C58" s="113"/>
+      <c r="D58" s="113"/>
+      <c r="E58" s="113"/>
+      <c r="F58" s="113"/>
       <c r="G58" s="41" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A59" s="98" t="s">
+      <c r="A59" s="112" t="s">
         <v>42</v>
       </c>
-      <c r="B59" s="98"/>
-      <c r="C59" s="98"/>
-      <c r="D59" s="98"/>
-      <c r="E59" s="98"/>
-      <c r="F59" s="98"/>
+      <c r="B59" s="112"/>
+      <c r="C59" s="112"/>
+      <c r="D59" s="112"/>
+      <c r="E59" s="112"/>
+      <c r="F59" s="112"/>
       <c r="G59" s="55">
         <f>VLOOKUP(A59,A53:G57,7,FALSE)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="59.25" customHeight="1"/>
+    <row r="60" spans="1:7" ht="22.5" customHeight="1"/>
     <row r="61" spans="1:7" ht="26.25">
-      <c r="A61" s="106" t="s">
+      <c r="A61" s="117" t="s">
         <v>76</v>
       </c>
-      <c r="B61" s="106"/>
-      <c r="C61" s="106"/>
-      <c r="D61" s="106"/>
-      <c r="E61" s="106"/>
-      <c r="F61" s="106"/>
-      <c r="G61" s="106"/>
+      <c r="B61" s="117"/>
+      <c r="C61" s="117"/>
+      <c r="D61" s="117"/>
+      <c r="E61" s="117"/>
+      <c r="F61" s="117"/>
+      <c r="G61" s="117"/>
     </row>
     <row r="62" spans="1:7" ht="31.5">
       <c r="A62" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="B62" s="133" t="s">
+      <c r="B62" s="144" t="s">
         <v>17</v>
       </c>
-      <c r="C62" s="134"/>
-      <c r="D62" s="134"/>
-      <c r="E62" s="134"/>
-      <c r="F62" s="135"/>
+      <c r="C62" s="145"/>
+      <c r="D62" s="145"/>
+      <c r="E62" s="145"/>
+      <c r="F62" s="146"/>
       <c r="G62" s="54" t="s">
         <v>3</v>
       </c>
@@ -3148,13 +3153,13 @@
       <c r="A63" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="B63" s="166" t="s">
+      <c r="B63" s="190" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="167"/>
-      <c r="D63" s="167"/>
-      <c r="E63" s="167"/>
-      <c r="F63" s="168"/>
+      <c r="C63" s="191"/>
+      <c r="D63" s="191"/>
+      <c r="E63" s="191"/>
+      <c r="F63" s="192"/>
       <c r="G63" s="14" t="s">
         <v>126</v>
       </c>
@@ -3163,13 +3168,13 @@
       <c r="A64" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="B64" s="112" t="s">
+      <c r="B64" s="123" t="s">
         <v>52</v>
       </c>
-      <c r="C64" s="112"/>
-      <c r="D64" s="112"/>
-      <c r="E64" s="112"/>
-      <c r="F64" s="112"/>
+      <c r="C64" s="123"/>
+      <c r="D64" s="123"/>
+      <c r="E64" s="123"/>
+      <c r="F64" s="123"/>
       <c r="G64" s="42">
         <v>0</v>
       </c>
@@ -3178,13 +3183,13 @@
       <c r="A65" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B65" s="136" t="s">
+      <c r="B65" s="147" t="s">
         <v>53</v>
       </c>
-      <c r="C65" s="136"/>
-      <c r="D65" s="136"/>
-      <c r="E65" s="136"/>
-      <c r="F65" s="136"/>
+      <c r="C65" s="147"/>
+      <c r="D65" s="147"/>
+      <c r="E65" s="147"/>
+      <c r="F65" s="147"/>
       <c r="G65" s="13">
         <v>4</v>
       </c>
@@ -3193,54 +3198,54 @@
       <c r="A66" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="B66" s="112" t="s">
+      <c r="B66" s="123" t="s">
         <v>54</v>
       </c>
-      <c r="C66" s="112"/>
-      <c r="D66" s="112"/>
-      <c r="E66" s="112"/>
-      <c r="F66" s="112"/>
+      <c r="C66" s="123"/>
+      <c r="D66" s="123"/>
+      <c r="E66" s="123"/>
+      <c r="F66" s="123"/>
       <c r="G66" s="42">
         <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="41.25" customHeight="1">
-      <c r="A67" s="129" t="s">
+      <c r="A67" s="140" t="s">
         <v>65</v>
       </c>
-      <c r="B67" s="130"/>
-      <c r="C67" s="130"/>
-      <c r="D67" s="130"/>
-      <c r="E67" s="130"/>
-      <c r="F67" s="131"/>
+      <c r="B67" s="141"/>
+      <c r="C67" s="141"/>
+      <c r="D67" s="141"/>
+      <c r="E67" s="141"/>
+      <c r="F67" s="142"/>
       <c r="G67" s="50" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="68" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A68" s="98" t="s">
-        <v>50</v>
-      </c>
-      <c r="B68" s="98"/>
-      <c r="C68" s="98"/>
-      <c r="D68" s="98"/>
-      <c r="E68" s="98"/>
-      <c r="F68" s="98"/>
-      <c r="G68" s="55">
+      <c r="A68" s="150" t="s">
+        <v>126</v>
+      </c>
+      <c r="B68" s="151"/>
+      <c r="C68" s="151"/>
+      <c r="D68" s="151"/>
+      <c r="E68" s="151"/>
+      <c r="F68" s="152"/>
+      <c r="G68" s="55" t="str">
         <f>VLOOKUP(A68,A63:G66,7,FALSE)</f>
-        <v>0</v>
+        <v>-</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="27.75">
-      <c r="A71" s="132" t="s">
+      <c r="A71" s="143" t="s">
         <v>75</v>
       </c>
-      <c r="B71" s="132"/>
-      <c r="C71" s="132"/>
-      <c r="D71" s="132"/>
-      <c r="E71" s="132"/>
-      <c r="F71" s="132"/>
-      <c r="G71" s="132"/>
+      <c r="B71" s="143"/>
+      <c r="C71" s="143"/>
+      <c r="D71" s="143"/>
+      <c r="E71" s="143"/>
+      <c r="F71" s="143"/>
+      <c r="G71" s="143"/>
     </row>
     <row r="72" spans="1:7" ht="51">
       <c r="A72" s="53" t="s">
@@ -3249,12 +3254,12 @@
       <c r="B72" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="C72" s="133" t="s">
+      <c r="C72" s="144" t="s">
         <v>60</v>
       </c>
-      <c r="D72" s="134"/>
-      <c r="E72" s="134"/>
-      <c r="F72" s="135"/>
+      <c r="D72" s="145"/>
+      <c r="E72" s="145"/>
+      <c r="F72" s="146"/>
       <c r="G72" s="54" t="s">
         <v>3</v>
       </c>
@@ -3266,12 +3271,12 @@
       <c r="B73" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="C73" s="166" t="s">
+      <c r="C73" s="190" t="s">
         <v>126</v>
       </c>
-      <c r="D73" s="167"/>
-      <c r="E73" s="167"/>
-      <c r="F73" s="168"/>
+      <c r="D73" s="191"/>
+      <c r="E73" s="191"/>
+      <c r="F73" s="192"/>
       <c r="G73" s="14" t="s">
         <v>126</v>
       </c>
@@ -3283,12 +3288,12 @@
       <c r="B74" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C74" s="112" t="s">
+      <c r="C74" s="123" t="s">
         <v>61</v>
       </c>
-      <c r="D74" s="112"/>
-      <c r="E74" s="112"/>
-      <c r="F74" s="112"/>
+      <c r="D74" s="123"/>
+      <c r="E74" s="123"/>
+      <c r="F74" s="123"/>
       <c r="G74" s="42">
         <v>0</v>
       </c>
@@ -3300,12 +3305,12 @@
       <c r="B75" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C75" s="136" t="s">
+      <c r="C75" s="147" t="s">
         <v>62</v>
       </c>
-      <c r="D75" s="136"/>
-      <c r="E75" s="136"/>
-      <c r="F75" s="136"/>
+      <c r="D75" s="147"/>
+      <c r="E75" s="147"/>
+      <c r="F75" s="147"/>
       <c r="G75" s="13">
         <v>4</v>
       </c>
@@ -3317,77 +3322,77 @@
       <c r="B76" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C76" s="112" t="s">
+      <c r="C76" s="123" t="s">
         <v>63</v>
       </c>
-      <c r="D76" s="112"/>
-      <c r="E76" s="112"/>
-      <c r="F76" s="112"/>
+      <c r="D76" s="123"/>
+      <c r="E76" s="123"/>
+      <c r="F76" s="123"/>
       <c r="G76" s="42">
         <v>6</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="39" customHeight="1">
-      <c r="A77" s="151" t="s">
+      <c r="A77" s="164" t="s">
         <v>66</v>
       </c>
-      <c r="B77" s="151"/>
-      <c r="C77" s="151"/>
-      <c r="D77" s="151"/>
-      <c r="E77" s="151"/>
-      <c r="F77" s="151"/>
+      <c r="B77" s="164"/>
+      <c r="C77" s="164"/>
+      <c r="D77" s="164"/>
+      <c r="E77" s="164"/>
+      <c r="F77" s="164"/>
       <c r="G77" s="43" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="78" spans="1:7" s="56" customFormat="1" ht="26.25">
-      <c r="A78" s="98">
-        <v>2</v>
-      </c>
-      <c r="B78" s="98"/>
-      <c r="C78" s="98"/>
-      <c r="D78" s="98"/>
-      <c r="E78" s="98"/>
-      <c r="F78" s="98"/>
-      <c r="G78" s="55">
+      <c r="A78" s="150" t="s">
+        <v>126</v>
+      </c>
+      <c r="B78" s="151"/>
+      <c r="C78" s="151"/>
+      <c r="D78" s="151"/>
+      <c r="E78" s="151"/>
+      <c r="F78" s="152"/>
+      <c r="G78" s="55" t="str">
         <f>VLOOKUP(A78,A73:G76,7)</f>
-        <v>4</v>
+        <v>-</v>
       </c>
     </row>
     <row r="80" spans="1:7" hidden="1"/>
     <row r="81" spans="1:7" ht="30">
-      <c r="A81" s="113" t="s">
+      <c r="A81" s="124" t="s">
         <v>74</v>
       </c>
-      <c r="B81" s="113"/>
-      <c r="C81" s="113"/>
-      <c r="D81" s="113"/>
-      <c r="E81" s="113"/>
-      <c r="F81" s="113"/>
-      <c r="G81" s="113"/>
+      <c r="B81" s="124"/>
+      <c r="C81" s="124"/>
+      <c r="D81" s="124"/>
+      <c r="E81" s="124"/>
+      <c r="F81" s="124"/>
+      <c r="G81" s="124"/>
     </row>
     <row r="82" spans="1:7" ht="42" customHeight="1">
-      <c r="A82" s="139" t="s">
+      <c r="A82" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="B82" s="139"/>
-      <c r="C82" s="139"/>
-      <c r="D82" s="139"/>
-      <c r="E82" s="139"/>
-      <c r="F82" s="139" t="s">
+      <c r="B82" s="153"/>
+      <c r="C82" s="153"/>
+      <c r="D82" s="153"/>
+      <c r="E82" s="153"/>
+      <c r="F82" s="153" t="s">
         <v>131</v>
       </c>
-      <c r="G82" s="139"/>
+      <c r="G82" s="153"/>
     </row>
     <row r="83" spans="1:7" ht="15" customHeight="1">
-      <c r="A83" s="142">
+      <c r="A83" s="155">
         <f>SUM(G29,G38,G59,G68,G78)</f>
-        <v>4</v>
-      </c>
-      <c r="B83" s="143"/>
-      <c r="C83" s="143"/>
-      <c r="D83" s="143"/>
-      <c r="E83" s="144"/>
+        <v>0</v>
+      </c>
+      <c r="B83" s="156"/>
+      <c r="C83" s="156"/>
+      <c r="D83" s="156"/>
+      <c r="E83" s="157"/>
       <c r="F83" s="12" t="s">
         <v>68</v>
       </c>
@@ -3396,11 +3401,11 @@
       </c>
     </row>
     <row r="84" spans="1:7" ht="15" customHeight="1">
-      <c r="A84" s="145"/>
-      <c r="B84" s="146"/>
-      <c r="C84" s="146"/>
-      <c r="D84" s="146"/>
-      <c r="E84" s="147"/>
+      <c r="A84" s="158"/>
+      <c r="B84" s="159"/>
+      <c r="C84" s="159"/>
+      <c r="D84" s="159"/>
+      <c r="E84" s="160"/>
       <c r="F84" s="19" t="s">
         <v>69</v>
       </c>
@@ -3409,11 +3414,11 @@
       </c>
     </row>
     <row r="85" spans="1:7" ht="15" customHeight="1">
-      <c r="A85" s="148"/>
-      <c r="B85" s="149"/>
-      <c r="C85" s="149"/>
-      <c r="D85" s="149"/>
-      <c r="E85" s="150"/>
+      <c r="A85" s="161"/>
+      <c r="B85" s="162"/>
+      <c r="C85" s="162"/>
+      <c r="D85" s="162"/>
+      <c r="E85" s="163"/>
       <c r="F85" s="12" t="s">
         <v>70</v>
       </c>
@@ -3422,436 +3427,436 @@
       </c>
     </row>
     <row r="86" spans="1:7" ht="44.25" customHeight="1">
-      <c r="A86" s="141" t="s">
+      <c r="A86" s="154" t="s">
         <v>72</v>
       </c>
-      <c r="B86" s="141"/>
-      <c r="C86" s="141"/>
-      <c r="D86" s="141"/>
-      <c r="E86" s="141"/>
-      <c r="F86" s="140" t="str">
+      <c r="B86" s="154"/>
+      <c r="C86" s="154"/>
+      <c r="D86" s="154"/>
+      <c r="E86" s="154"/>
+      <c r="F86" s="193" t="str">
         <f>IF(A83="-","-",IF(A83&lt;=14,G83,IF(AND(A83&gt;=15,A83&lt;=30),G84,G85)))</f>
         <v>Χαμηλό</v>
       </c>
-      <c r="G86" s="140"/>
+      <c r="G86" s="193"/>
     </row>
     <row r="89" spans="1:7" ht="26.25">
-      <c r="A89" s="106" t="s">
+      <c r="A89" s="117" t="s">
         <v>108</v>
       </c>
-      <c r="B89" s="106"/>
-      <c r="C89" s="106"/>
-      <c r="D89" s="106"/>
-      <c r="E89" s="106"/>
-      <c r="F89" s="106"/>
-      <c r="G89" s="106"/>
+      <c r="B89" s="117"/>
+      <c r="C89" s="117"/>
+      <c r="D89" s="117"/>
+      <c r="E89" s="117"/>
+      <c r="F89" s="117"/>
+      <c r="G89" s="117"/>
     </row>
     <row r="90" spans="1:7">
-      <c r="A90" s="152" t="s">
+      <c r="A90" s="167" t="s">
         <v>127</v>
       </c>
-      <c r="B90" s="152"/>
-      <c r="C90" s="152"/>
-      <c r="D90" s="152"/>
-      <c r="E90" s="152" t="s">
+      <c r="B90" s="167"/>
+      <c r="C90" s="167"/>
+      <c r="D90" s="167"/>
+      <c r="E90" s="167" t="s">
         <v>103</v>
       </c>
-      <c r="F90" s="152"/>
-      <c r="G90" s="152"/>
+      <c r="F90" s="167"/>
+      <c r="G90" s="167"/>
     </row>
     <row r="91" spans="1:7">
-      <c r="A91" s="156" t="s">
+      <c r="A91" s="169" t="s">
         <v>126</v>
       </c>
-      <c r="B91" s="157"/>
-      <c r="C91" s="157"/>
-      <c r="D91" s="158"/>
-      <c r="E91" s="156" t="s">
+      <c r="B91" s="170"/>
+      <c r="C91" s="170"/>
+      <c r="D91" s="171"/>
+      <c r="E91" s="169" t="s">
         <v>126</v>
       </c>
-      <c r="F91" s="157"/>
-      <c r="G91" s="158"/>
+      <c r="F91" s="170"/>
+      <c r="G91" s="171"/>
     </row>
     <row r="92" spans="1:7">
-      <c r="A92" s="110" t="s">
+      <c r="A92" s="121" t="s">
         <v>34</v>
       </c>
-      <c r="B92" s="110"/>
-      <c r="C92" s="110"/>
-      <c r="D92" s="110"/>
-      <c r="E92" s="110" t="s">
+      <c r="B92" s="121"/>
+      <c r="C92" s="121"/>
+      <c r="D92" s="121"/>
+      <c r="E92" s="121" t="s">
         <v>132</v>
       </c>
-      <c r="F92" s="110"/>
-      <c r="G92" s="110"/>
+      <c r="F92" s="121"/>
+      <c r="G92" s="121"/>
     </row>
     <row r="93" spans="1:7">
-      <c r="A93" s="153" t="s">
+      <c r="A93" s="165" t="s">
         <v>35</v>
       </c>
-      <c r="B93" s="153"/>
-      <c r="C93" s="153"/>
-      <c r="D93" s="153"/>
-      <c r="E93" s="153" t="s">
+      <c r="B93" s="165"/>
+      <c r="C93" s="165"/>
+      <c r="D93" s="165"/>
+      <c r="E93" s="165" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="153"/>
-      <c r="G93" s="153"/>
+      <c r="F93" s="165"/>
+      <c r="G93" s="165"/>
     </row>
     <row r="94" spans="1:7">
-      <c r="A94" s="112" t="s">
+      <c r="A94" s="123" t="s">
         <v>36</v>
       </c>
-      <c r="B94" s="112"/>
-      <c r="C94" s="112"/>
-      <c r="D94" s="112"/>
-      <c r="E94" s="110" t="s">
+      <c r="B94" s="123"/>
+      <c r="C94" s="123"/>
+      <c r="D94" s="123"/>
+      <c r="E94" s="121" t="s">
         <v>106</v>
       </c>
-      <c r="F94" s="110"/>
-      <c r="G94" s="110"/>
+      <c r="F94" s="121"/>
+      <c r="G94" s="121"/>
     </row>
     <row r="95" spans="1:7" ht="15.75">
-      <c r="A95" s="154" t="s">
+      <c r="A95" s="166" t="s">
         <v>107</v>
       </c>
-      <c r="B95" s="154"/>
-      <c r="C95" s="154"/>
-      <c r="D95" s="154"/>
-      <c r="E95" s="154"/>
-      <c r="F95" s="154"/>
-      <c r="G95" s="154"/>
+      <c r="B95" s="166"/>
+      <c r="C95" s="166"/>
+      <c r="D95" s="166"/>
+      <c r="E95" s="166"/>
+      <c r="F95" s="166"/>
+      <c r="G95" s="166"/>
     </row>
     <row r="96" spans="1:7" ht="37.5" customHeight="1">
-      <c r="A96" s="99" t="s">
+      <c r="A96" s="113" t="s">
         <v>129</v>
       </c>
-      <c r="B96" s="99"/>
-      <c r="C96" s="99"/>
-      <c r="D96" s="99"/>
-      <c r="E96" s="161" t="s">
+      <c r="B96" s="113"/>
+      <c r="C96" s="113"/>
+      <c r="D96" s="113"/>
+      <c r="E96" s="187" t="s">
         <v>103</v>
       </c>
-      <c r="F96" s="161"/>
-      <c r="G96" s="161"/>
+      <c r="F96" s="187"/>
+      <c r="G96" s="187"/>
     </row>
     <row r="97" spans="1:7" ht="55.5" customHeight="1">
-      <c r="A97" s="155" t="str">
+      <c r="A97" s="168" t="str">
         <f>F86</f>
         <v>Χαμηλό</v>
       </c>
-      <c r="B97" s="155"/>
-      <c r="C97" s="155"/>
-      <c r="D97" s="155"/>
-      <c r="E97" s="162" t="str">
+      <c r="B97" s="168"/>
+      <c r="C97" s="168"/>
+      <c r="D97" s="168"/>
+      <c r="E97" s="188" t="str">
         <f>VLOOKUP(A97,A91:G94,5,FALSE)</f>
         <v>Δεν πραγματοποιούνται έλεγχοι</v>
       </c>
-      <c r="F97" s="162"/>
-      <c r="G97" s="162"/>
+      <c r="F97" s="188"/>
+      <c r="G97" s="188"/>
     </row>
     <row r="100" spans="1:7" ht="24">
-      <c r="A100" s="165" t="s">
+      <c r="A100" s="189" t="s">
         <v>134</v>
       </c>
-      <c r="B100" s="165"/>
-      <c r="C100" s="165"/>
-      <c r="D100" s="165"/>
-      <c r="E100" s="165"/>
-      <c r="F100" s="165"/>
-      <c r="G100" s="165"/>
+      <c r="B100" s="189"/>
+      <c r="C100" s="189"/>
+      <c r="D100" s="189"/>
+      <c r="E100" s="189"/>
+      <c r="F100" s="189"/>
+      <c r="G100" s="189"/>
     </row>
     <row r="101" spans="1:7" ht="26.25">
-      <c r="A101" s="106" t="s">
+      <c r="A101" s="117" t="s">
         <v>73</v>
       </c>
-      <c r="B101" s="106"/>
-      <c r="C101" s="106"/>
-      <c r="D101" s="106"/>
-      <c r="E101" s="106"/>
-      <c r="F101" s="106"/>
-      <c r="G101" s="106"/>
+      <c r="B101" s="117"/>
+      <c r="C101" s="117"/>
+      <c r="D101" s="117"/>
+      <c r="E101" s="117"/>
+      <c r="F101" s="117"/>
+      <c r="G101" s="117"/>
     </row>
     <row r="102" spans="1:7" ht="24.75" customHeight="1">
-      <c r="A102" s="159" t="s">
+      <c r="A102" s="186" t="s">
         <v>71</v>
       </c>
-      <c r="B102" s="159"/>
-      <c r="C102" s="159"/>
-      <c r="D102" s="159"/>
-      <c r="E102" s="159"/>
-      <c r="F102" s="159"/>
+      <c r="B102" s="186"/>
+      <c r="C102" s="186"/>
+      <c r="D102" s="186"/>
+      <c r="E102" s="186"/>
+      <c r="F102" s="186"/>
       <c r="G102" s="26" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="15.75">
-      <c r="A103" s="159" t="s">
+      <c r="A103" s="72" t="s">
         <v>126</v>
       </c>
-      <c r="B103" s="159"/>
-      <c r="C103" s="159"/>
-      <c r="D103" s="159"/>
-      <c r="E103" s="159"/>
-      <c r="F103" s="159"/>
+      <c r="B103" s="73"/>
+      <c r="C103" s="73"/>
+      <c r="D103" s="73"/>
+      <c r="E103" s="73"/>
+      <c r="F103" s="74"/>
       <c r="G103" s="26" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="104" spans="1:7">
-      <c r="A104" s="110" t="s">
+      <c r="A104" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="B104" s="110"/>
-      <c r="C104" s="110"/>
-      <c r="D104" s="110"/>
-      <c r="E104" s="110"/>
-      <c r="F104" s="110"/>
+      <c r="B104" s="76"/>
+      <c r="C104" s="76"/>
+      <c r="D104" s="76"/>
+      <c r="E104" s="76"/>
+      <c r="F104" s="77"/>
       <c r="G104" s="42">
         <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:7">
-      <c r="A105" s="160" t="s">
+      <c r="A105" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="B105" s="160"/>
-      <c r="C105" s="160"/>
-      <c r="D105" s="160"/>
-      <c r="E105" s="160"/>
-      <c r="F105" s="160"/>
+      <c r="B105" s="79"/>
+      <c r="C105" s="79"/>
+      <c r="D105" s="79"/>
+      <c r="E105" s="79"/>
+      <c r="F105" s="80"/>
       <c r="G105" s="24">
         <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:7">
-      <c r="A106" s="110" t="s">
+      <c r="A106" s="75" t="s">
         <v>51</v>
       </c>
-      <c r="B106" s="110"/>
-      <c r="C106" s="110"/>
-      <c r="D106" s="110"/>
-      <c r="E106" s="110"/>
-      <c r="F106" s="110"/>
+      <c r="B106" s="76"/>
+      <c r="C106" s="76"/>
+      <c r="D106" s="76"/>
+      <c r="E106" s="76"/>
+      <c r="F106" s="77"/>
       <c r="G106" s="42">
         <v>12</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="47.25" customHeight="1">
-      <c r="A107" s="205" t="s">
+      <c r="A107" s="185" t="s">
         <v>81</v>
       </c>
-      <c r="B107" s="205"/>
-      <c r="C107" s="205"/>
-      <c r="D107" s="205"/>
-      <c r="E107" s="205"/>
-      <c r="F107" s="205"/>
+      <c r="B107" s="185"/>
+      <c r="C107" s="185"/>
+      <c r="D107" s="185"/>
+      <c r="E107" s="185"/>
+      <c r="F107" s="185"/>
       <c r="G107" s="27" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="33.75">
-      <c r="A108" s="98" t="s">
+      <c r="A108" s="150" t="s">
         <v>126</v>
       </c>
-      <c r="B108" s="98"/>
-      <c r="C108" s="98"/>
-      <c r="D108" s="98"/>
-      <c r="E108" s="98"/>
-      <c r="F108" s="98"/>
+      <c r="B108" s="151"/>
+      <c r="C108" s="151"/>
+      <c r="D108" s="151"/>
+      <c r="E108" s="151"/>
+      <c r="F108" s="152"/>
       <c r="G108" s="40" t="str">
         <f>VLOOKUP(A108,A103:G106,7,FALSE)</f>
         <v>-</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="26.25">
-      <c r="A112" s="106" t="s">
+      <c r="A112" s="117" t="s">
         <v>77</v>
       </c>
-      <c r="B112" s="106"/>
-      <c r="C112" s="106"/>
-      <c r="D112" s="106"/>
-      <c r="E112" s="106"/>
-      <c r="F112" s="106"/>
-      <c r="G112" s="106"/>
+      <c r="B112" s="117"/>
+      <c r="C112" s="117"/>
+      <c r="D112" s="117"/>
+      <c r="E112" s="117"/>
+      <c r="F112" s="117"/>
+      <c r="G112" s="117"/>
     </row>
     <row r="113" spans="1:7" ht="27.75" customHeight="1">
-      <c r="A113" s="159" t="s">
+      <c r="A113" s="186" t="s">
         <v>77</v>
       </c>
-      <c r="B113" s="159"/>
-      <c r="C113" s="159"/>
-      <c r="D113" s="159"/>
-      <c r="E113" s="159"/>
-      <c r="F113" s="159"/>
+      <c r="B113" s="186"/>
+      <c r="C113" s="186"/>
+      <c r="D113" s="186"/>
+      <c r="E113" s="186"/>
+      <c r="F113" s="186"/>
       <c r="G113" s="26" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="15.75">
-      <c r="A114" s="159" t="s">
+      <c r="A114" s="72" t="s">
         <v>126</v>
       </c>
-      <c r="B114" s="159"/>
-      <c r="C114" s="159"/>
-      <c r="D114" s="159"/>
-      <c r="E114" s="159"/>
-      <c r="F114" s="159"/>
+      <c r="B114" s="73"/>
+      <c r="C114" s="73"/>
+      <c r="D114" s="73"/>
+      <c r="E114" s="73"/>
+      <c r="F114" s="74"/>
       <c r="G114" s="26" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="115" spans="1:7">
-      <c r="A115" s="110" t="s">
+      <c r="A115" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="B115" s="110"/>
-      <c r="C115" s="110"/>
-      <c r="D115" s="110"/>
-      <c r="E115" s="110"/>
-      <c r="F115" s="110"/>
+      <c r="B115" s="76"/>
+      <c r="C115" s="76"/>
+      <c r="D115" s="76"/>
+      <c r="E115" s="76"/>
+      <c r="F115" s="77"/>
       <c r="G115" s="42">
         <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:7">
-      <c r="A116" s="160" t="s">
+      <c r="A116" s="78" t="s">
         <v>79</v>
       </c>
-      <c r="B116" s="160"/>
-      <c r="C116" s="160"/>
-      <c r="D116" s="160"/>
-      <c r="E116" s="160"/>
-      <c r="F116" s="160"/>
+      <c r="B116" s="79"/>
+      <c r="C116" s="79"/>
+      <c r="D116" s="79"/>
+      <c r="E116" s="79"/>
+      <c r="F116" s="80"/>
       <c r="G116" s="24">
         <v>3</v>
       </c>
     </row>
     <row r="117" spans="1:7">
-      <c r="A117" s="110" t="s">
+      <c r="A117" s="75" t="s">
         <v>80</v>
       </c>
-      <c r="B117" s="110"/>
-      <c r="C117" s="110"/>
-      <c r="D117" s="110"/>
-      <c r="E117" s="110"/>
-      <c r="F117" s="110"/>
+      <c r="B117" s="76"/>
+      <c r="C117" s="76"/>
+      <c r="D117" s="76"/>
+      <c r="E117" s="76"/>
+      <c r="F117" s="77"/>
       <c r="G117" s="42">
         <v>6</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="18">
-      <c r="A118" s="201" t="s">
+      <c r="A118" s="184" t="s">
         <v>82</v>
       </c>
-      <c r="B118" s="201"/>
-      <c r="C118" s="201"/>
-      <c r="D118" s="201"/>
-      <c r="E118" s="201"/>
-      <c r="F118" s="201"/>
+      <c r="B118" s="184"/>
+      <c r="C118" s="184"/>
+      <c r="D118" s="184"/>
+      <c r="E118" s="184"/>
+      <c r="F118" s="184"/>
       <c r="G118" s="27" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="26.25">
-      <c r="A119" s="202" t="s">
+      <c r="A119" s="150" t="s">
         <v>126</v>
       </c>
-      <c r="B119" s="203"/>
-      <c r="C119" s="203"/>
-      <c r="D119" s="203"/>
-      <c r="E119" s="203"/>
-      <c r="F119" s="204"/>
+      <c r="B119" s="151"/>
+      <c r="C119" s="151"/>
+      <c r="D119" s="151"/>
+      <c r="E119" s="151"/>
+      <c r="F119" s="152"/>
       <c r="G119" s="55" t="str">
         <f>VLOOKUP(A119,A114:G117,7,FALSE)</f>
         <v>-</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="35.25" customHeight="1">
-      <c r="A122" s="193" t="s">
+      <c r="A122" s="176" t="s">
         <v>84</v>
       </c>
-      <c r="B122" s="193"/>
-      <c r="C122" s="193"/>
-      <c r="D122" s="193"/>
-      <c r="E122" s="193"/>
-      <c r="F122" s="193"/>
-      <c r="G122" s="193"/>
+      <c r="B122" s="176"/>
+      <c r="C122" s="176"/>
+      <c r="D122" s="176"/>
+      <c r="E122" s="176"/>
+      <c r="F122" s="176"/>
+      <c r="G122" s="176"/>
     </row>
     <row r="123" spans="1:7" ht="135" customHeight="1">
-      <c r="A123" s="139" t="s">
+      <c r="A123" s="153" t="s">
         <v>140</v>
       </c>
-      <c r="B123" s="139"/>
-      <c r="C123" s="139"/>
+      <c r="B123" s="153"/>
+      <c r="C123" s="153"/>
       <c r="D123" s="65" t="s">
         <v>94</v>
       </c>
-      <c r="E123" s="139" t="s">
+      <c r="E123" s="153" t="s">
         <v>85</v>
       </c>
-      <c r="F123" s="139"/>
+      <c r="F123" s="153"/>
       <c r="G123" s="59" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="15" customHeight="1">
-      <c r="A124" s="200" t="str">
+      <c r="A124" s="183" t="str">
         <f>IF(AND(G108="-",G119="-"),"-",IF(G119="-",SUM(A83,G108),SUM(A83,G108,G119)))</f>
         <v>-</v>
       </c>
-      <c r="B124" s="200"/>
-      <c r="C124" s="200"/>
+      <c r="B124" s="183"/>
+      <c r="C124" s="183"/>
       <c r="D124" s="63" t="s">
         <v>89</v>
       </c>
-      <c r="E124" s="194" t="s">
+      <c r="E124" s="177" t="s">
         <v>86</v>
       </c>
-      <c r="F124" s="195"/>
+      <c r="F124" s="178"/>
       <c r="G124" s="29" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="15" customHeight="1">
-      <c r="A125" s="200"/>
-      <c r="B125" s="200"/>
-      <c r="C125" s="200"/>
+      <c r="A125" s="183"/>
+      <c r="B125" s="183"/>
+      <c r="C125" s="183"/>
       <c r="D125" s="64" t="s">
         <v>90</v>
       </c>
-      <c r="E125" s="196" t="s">
+      <c r="E125" s="179" t="s">
         <v>87</v>
       </c>
-      <c r="F125" s="197"/>
+      <c r="F125" s="180"/>
       <c r="G125" s="31" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="15" customHeight="1">
-      <c r="A126" s="200"/>
-      <c r="B126" s="200"/>
-      <c r="C126" s="200"/>
+      <c r="A126" s="183"/>
+      <c r="B126" s="183"/>
+      <c r="C126" s="183"/>
       <c r="D126" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="E126" s="198" t="s">
+      <c r="E126" s="181" t="s">
         <v>88</v>
       </c>
-      <c r="F126" s="199"/>
+      <c r="F126" s="182"/>
       <c r="G126" s="29" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="53.25" customHeight="1">
-      <c r="A127" s="141" t="s">
+      <c r="A127" s="154" t="s">
         <v>93</v>
       </c>
-      <c r="B127" s="141"/>
-      <c r="C127" s="141"/>
-      <c r="D127" s="141"/>
-      <c r="E127" s="141"/>
-      <c r="F127" s="141"/>
+      <c r="B127" s="154"/>
+      <c r="C127" s="154"/>
+      <c r="D127" s="154"/>
+      <c r="E127" s="154"/>
+      <c r="F127" s="154"/>
       <c r="G127" s="62" t="str">
         <f>IF(A124="-","-",IF(G119="-",IF(A124&lt;=19,G124,IF(A124&gt;=40,G126,G125)),IF(A124&lt;=21,G124,IF(A124&gt;=44,G126,G125))))</f>
         <v>-</v>
@@ -3867,173 +3872,173 @@
       <c r="G128" s="61"/>
     </row>
     <row r="131" spans="1:7" ht="26.25">
-      <c r="A131" s="106" t="s">
+      <c r="A131" s="117" t="s">
         <v>139</v>
       </c>
-      <c r="B131" s="106"/>
-      <c r="C131" s="106"/>
-      <c r="D131" s="106"/>
-      <c r="E131" s="106"/>
-      <c r="F131" s="106"/>
-      <c r="G131" s="106"/>
+      <c r="B131" s="117"/>
+      <c r="C131" s="117"/>
+      <c r="D131" s="117"/>
+      <c r="E131" s="117"/>
+      <c r="F131" s="117"/>
+      <c r="G131" s="117"/>
     </row>
     <row r="132" spans="1:7">
-      <c r="A132" s="152" t="s">
+      <c r="A132" s="167" t="s">
         <v>128</v>
       </c>
-      <c r="B132" s="152"/>
-      <c r="C132" s="152"/>
-      <c r="D132" s="152"/>
-      <c r="E132" s="152" t="s">
+      <c r="B132" s="167"/>
+      <c r="C132" s="167"/>
+      <c r="D132" s="167"/>
+      <c r="E132" s="167" t="s">
         <v>103</v>
       </c>
-      <c r="F132" s="152"/>
-      <c r="G132" s="152"/>
+      <c r="F132" s="167"/>
+      <c r="G132" s="167"/>
     </row>
     <row r="133" spans="1:7">
-      <c r="A133" s="156" t="s">
+      <c r="A133" s="169" t="s">
         <v>126</v>
       </c>
-      <c r="B133" s="157"/>
-      <c r="C133" s="157"/>
-      <c r="D133" s="158"/>
-      <c r="E133" s="156" t="s">
+      <c r="B133" s="170"/>
+      <c r="C133" s="170"/>
+      <c r="D133" s="171"/>
+      <c r="E133" s="169" t="s">
         <v>126</v>
       </c>
-      <c r="F133" s="157"/>
-      <c r="G133" s="158"/>
+      <c r="F133" s="170"/>
+      <c r="G133" s="171"/>
     </row>
     <row r="134" spans="1:7">
-      <c r="A134" s="110" t="s">
+      <c r="A134" s="121" t="s">
         <v>34</v>
       </c>
-      <c r="B134" s="110"/>
-      <c r="C134" s="110"/>
-      <c r="D134" s="110"/>
-      <c r="E134" s="110" t="s">
+      <c r="B134" s="121"/>
+      <c r="C134" s="121"/>
+      <c r="D134" s="121"/>
+      <c r="E134" s="121" t="s">
         <v>104</v>
       </c>
-      <c r="F134" s="110"/>
-      <c r="G134" s="110"/>
+      <c r="F134" s="121"/>
+      <c r="G134" s="121"/>
     </row>
     <row r="135" spans="1:7">
-      <c r="A135" s="153" t="s">
+      <c r="A135" s="165" t="s">
         <v>35</v>
       </c>
-      <c r="B135" s="153"/>
-      <c r="C135" s="153"/>
-      <c r="D135" s="153"/>
-      <c r="E135" s="153" t="s">
+      <c r="B135" s="165"/>
+      <c r="C135" s="165"/>
+      <c r="D135" s="165"/>
+      <c r="E135" s="165" t="s">
         <v>105</v>
       </c>
-      <c r="F135" s="153"/>
-      <c r="G135" s="153"/>
+      <c r="F135" s="165"/>
+      <c r="G135" s="165"/>
     </row>
     <row r="136" spans="1:7">
-      <c r="A136" s="110" t="s">
+      <c r="A136" s="121" t="s">
         <v>36</v>
       </c>
-      <c r="B136" s="110"/>
-      <c r="C136" s="110"/>
-      <c r="D136" s="110"/>
-      <c r="E136" s="110" t="s">
+      <c r="B136" s="121"/>
+      <c r="C136" s="121"/>
+      <c r="D136" s="121"/>
+      <c r="E136" s="121" t="s">
         <v>106</v>
       </c>
-      <c r="F136" s="110"/>
-      <c r="G136" s="110"/>
+      <c r="F136" s="121"/>
+      <c r="G136" s="121"/>
     </row>
     <row r="137" spans="1:7" ht="15.75">
-      <c r="A137" s="154" t="s">
+      <c r="A137" s="166" t="s">
         <v>107</v>
       </c>
-      <c r="B137" s="154"/>
-      <c r="C137" s="154"/>
-      <c r="D137" s="154"/>
-      <c r="E137" s="154"/>
-      <c r="F137" s="154"/>
-      <c r="G137" s="154"/>
+      <c r="B137" s="166"/>
+      <c r="C137" s="166"/>
+      <c r="D137" s="166"/>
+      <c r="E137" s="166"/>
+      <c r="F137" s="166"/>
+      <c r="G137" s="166"/>
     </row>
     <row r="138" spans="1:7" ht="60" customHeight="1">
-      <c r="A138" s="99" t="s">
+      <c r="A138" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="B138" s="99"/>
-      <c r="C138" s="99"/>
-      <c r="D138" s="99"/>
-      <c r="E138" s="161" t="s">
+      <c r="B138" s="113"/>
+      <c r="C138" s="113"/>
+      <c r="D138" s="113"/>
+      <c r="E138" s="187" t="s">
         <v>103</v>
       </c>
-      <c r="F138" s="161"/>
-      <c r="G138" s="161"/>
+      <c r="F138" s="187"/>
+      <c r="G138" s="187"/>
     </row>
     <row r="139" spans="1:7" ht="54.75" customHeight="1">
-      <c r="A139" s="169" t="str">
+      <c r="A139" s="206" t="str">
         <f>G127</f>
         <v>-</v>
       </c>
-      <c r="B139" s="169"/>
-      <c r="C139" s="169"/>
-      <c r="D139" s="169"/>
-      <c r="E139" s="180" t="str">
+      <c r="B139" s="206"/>
+      <c r="C139" s="206"/>
+      <c r="D139" s="206"/>
+      <c r="E139" s="217" t="str">
         <f>VLOOKUP(A139,A133:G136,5,FALSE)</f>
         <v>-</v>
       </c>
-      <c r="F139" s="180"/>
-      <c r="G139" s="180"/>
+      <c r="F139" s="217"/>
+      <c r="G139" s="217"/>
     </row>
     <row r="142" spans="1:7" ht="15.75" thickBot="1"/>
     <row r="143" spans="1:7" ht="24" customHeight="1" thickBot="1">
-      <c r="A143" s="187" t="s">
+      <c r="A143" s="200" t="s">
         <v>141</v>
       </c>
-      <c r="B143" s="188"/>
-      <c r="C143" s="188"/>
-      <c r="D143" s="188"/>
-      <c r="E143" s="189">
+      <c r="B143" s="201"/>
+      <c r="C143" s="201"/>
+      <c r="D143" s="201"/>
+      <c r="E143" s="202">
         <f>E4</f>
         <v>0</v>
       </c>
-      <c r="F143" s="189"/>
-      <c r="G143" s="190"/>
+      <c r="F143" s="202"/>
+      <c r="G143" s="203"/>
     </row>
     <row r="144" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A144" s="170" t="s">
+      <c r="A144" s="207" t="s">
         <v>135</v>
       </c>
-      <c r="B144" s="171"/>
-      <c r="C144" s="171"/>
-      <c r="D144" s="171"/>
-      <c r="E144" s="171"/>
-      <c r="F144" s="171"/>
-      <c r="G144" s="172"/>
+      <c r="B144" s="208"/>
+      <c r="C144" s="208"/>
+      <c r="D144" s="208"/>
+      <c r="E144" s="208"/>
+      <c r="F144" s="208"/>
+      <c r="G144" s="209"/>
     </row>
     <row r="145" spans="1:7" ht="37.5" customHeight="1" thickBot="1">
-      <c r="A145" s="173" t="s">
+      <c r="A145" s="210" t="s">
         <v>136</v>
       </c>
-      <c r="B145" s="174"/>
-      <c r="C145" s="174"/>
-      <c r="D145" s="174"/>
-      <c r="E145" s="175" t="s">
+      <c r="B145" s="211"/>
+      <c r="C145" s="211"/>
+      <c r="D145" s="211"/>
+      <c r="E145" s="212" t="s">
         <v>137</v>
       </c>
-      <c r="F145" s="175"/>
-      <c r="G145" s="176"/>
+      <c r="F145" s="212"/>
+      <c r="G145" s="213"/>
     </row>
     <row r="146" spans="1:7" ht="30.75" customHeight="1" thickBot="1">
-      <c r="A146" s="163">
+      <c r="A146" s="204">
         <f>G4</f>
         <v>0</v>
       </c>
-      <c r="B146" s="164"/>
-      <c r="C146" s="164"/>
-      <c r="D146" s="164"/>
-      <c r="E146" s="177">
+      <c r="B146" s="205"/>
+      <c r="C146" s="205"/>
+      <c r="D146" s="205"/>
+      <c r="E146" s="214">
         <f>G4</f>
         <v>0</v>
       </c>
-      <c r="F146" s="178"/>
-      <c r="G146" s="179"/>
+      <c r="F146" s="215"/>
+      <c r="G146" s="216"/>
     </row>
     <row r="147" spans="1:7" ht="14.25" customHeight="1">
       <c r="A147" s="66" t="s">
@@ -4042,80 +4047,58 @@
       <c r="B147" s="67"/>
       <c r="C147" s="67"/>
       <c r="D147" s="67"/>
-      <c r="E147" s="181" t="s">
+      <c r="E147" s="194" t="s">
         <v>144</v>
       </c>
-      <c r="F147" s="181"/>
-      <c r="G147" s="182"/>
+      <c r="F147" s="194"/>
+      <c r="G147" s="195"/>
     </row>
     <row r="148" spans="1:7" ht="14.25" customHeight="1">
       <c r="A148" s="68"/>
       <c r="B148" s="69"/>
       <c r="C148" s="69"/>
       <c r="D148" s="69"/>
-      <c r="E148" s="183"/>
-      <c r="F148" s="183"/>
-      <c r="G148" s="184"/>
+      <c r="E148" s="196"/>
+      <c r="F148" s="196"/>
+      <c r="G148" s="197"/>
     </row>
     <row r="149" spans="1:7" ht="14.25" customHeight="1">
       <c r="A149" s="68"/>
       <c r="B149" s="69"/>
       <c r="C149" s="69"/>
       <c r="D149" s="69"/>
-      <c r="E149" s="183"/>
-      <c r="F149" s="183"/>
-      <c r="G149" s="184"/>
+      <c r="E149" s="196"/>
+      <c r="F149" s="196"/>
+      <c r="G149" s="197"/>
     </row>
     <row r="150" spans="1:7" ht="14.25" customHeight="1">
       <c r="A150" s="68"/>
       <c r="B150" s="69"/>
       <c r="C150" s="69"/>
       <c r="D150" s="69"/>
-      <c r="E150" s="183"/>
-      <c r="F150" s="183"/>
-      <c r="G150" s="184"/>
+      <c r="E150" s="196"/>
+      <c r="F150" s="196"/>
+      <c r="G150" s="197"/>
     </row>
     <row r="151" spans="1:7" ht="15" customHeight="1" thickBot="1">
       <c r="A151" s="70"/>
       <c r="B151" s="71"/>
       <c r="C151" s="71"/>
       <c r="D151" s="71"/>
-      <c r="E151" s="185"/>
-      <c r="F151" s="185"/>
-      <c r="G151" s="186"/>
+      <c r="E151" s="198"/>
+      <c r="F151" s="198"/>
+      <c r="G151" s="199"/>
     </row>
   </sheetData>
-  <mergeCells count="160">
+  <mergeCells count="147">
     <mergeCell ref="E147:G151"/>
     <mergeCell ref="A143:D143"/>
     <mergeCell ref="E143:G143"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="A122:G122"/>
-    <mergeCell ref="E123:F123"/>
-    <mergeCell ref="E124:F124"/>
-    <mergeCell ref="E125:F125"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="A123:C123"/>
-    <mergeCell ref="A124:C126"/>
     <mergeCell ref="A127:F127"/>
     <mergeCell ref="E136:G136"/>
     <mergeCell ref="A133:D133"/>
     <mergeCell ref="E133:G133"/>
-    <mergeCell ref="A114:F114"/>
-    <mergeCell ref="A115:F115"/>
-    <mergeCell ref="A116:F116"/>
-    <mergeCell ref="A117:F117"/>
-    <mergeCell ref="A118:F118"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A107:F107"/>
-    <mergeCell ref="A108:F108"/>
     <mergeCell ref="A146:D146"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="C73:F73"/>
     <mergeCell ref="A139:D139"/>
     <mergeCell ref="A144:G144"/>
     <mergeCell ref="A145:D145"/>
@@ -4126,24 +4109,30 @@
     <mergeCell ref="A131:G131"/>
     <mergeCell ref="A132:D132"/>
     <mergeCell ref="A134:D134"/>
-    <mergeCell ref="A135:D135"/>
-    <mergeCell ref="A136:D136"/>
-    <mergeCell ref="A137:G137"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="C73:F73"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="A108:F108"/>
     <mergeCell ref="A138:D138"/>
     <mergeCell ref="E132:G132"/>
     <mergeCell ref="E134:G134"/>
     <mergeCell ref="E135:G135"/>
     <mergeCell ref="A100:G100"/>
+    <mergeCell ref="A118:F118"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A107:F107"/>
     <mergeCell ref="A113:F113"/>
     <mergeCell ref="A112:G112"/>
     <mergeCell ref="A102:F102"/>
-    <mergeCell ref="A103:F103"/>
-    <mergeCell ref="A104:F104"/>
-    <mergeCell ref="A105:F105"/>
-    <mergeCell ref="A106:F106"/>
     <mergeCell ref="E96:G96"/>
     <mergeCell ref="E97:G97"/>
     <mergeCell ref="A101:G101"/>
+    <mergeCell ref="A135:D135"/>
+    <mergeCell ref="A136:D136"/>
+    <mergeCell ref="A137:G137"/>
     <mergeCell ref="A89:G89"/>
     <mergeCell ref="A90:D90"/>
     <mergeCell ref="A92:D92"/>
@@ -4158,8 +4147,13 @@
     <mergeCell ref="E93:G93"/>
     <mergeCell ref="E94:G94"/>
     <mergeCell ref="E91:G91"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="A122:G122"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="A123:C123"/>
+    <mergeCell ref="A124:C126"/>
     <mergeCell ref="A82:E82"/>
     <mergeCell ref="A86:E86"/>
     <mergeCell ref="A83:E85"/>
@@ -4171,7 +4165,6 @@
     <mergeCell ref="A77:F77"/>
     <mergeCell ref="A78:F78"/>
     <mergeCell ref="A67:F67"/>
-    <mergeCell ref="A68:F68"/>
     <mergeCell ref="A61:G61"/>
     <mergeCell ref="A71:G71"/>
     <mergeCell ref="A51:G51"/>
@@ -4185,12 +4178,9 @@
     <mergeCell ref="C56:F56"/>
     <mergeCell ref="C57:F57"/>
     <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A57:B57"/>
     <mergeCell ref="C52:F52"/>
     <mergeCell ref="C53:F53"/>
+    <mergeCell ref="A68:F68"/>
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="A46:D46"/>
@@ -4212,7 +4202,6 @@
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="E16:G16"/>
@@ -4221,7 +4210,6 @@
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:G6"/>
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="B21:F21"/>
@@ -4246,29 +4234,45 @@
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A29">
       <formula1>A22:A27</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A38 A68:F68 A78:F78 A119:F119 A108:F108">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A38">
       <formula1>A33:A36</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A59:F59">
-      <formula1>A53:A57</formula1>
+      <formula1>PLITHOS</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A134:A136 A92:A94">
       <formula1>$A$3:$A$5</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A68:F68">
+      <formula1>ktiriaki_pol</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A108:F108">
+      <formula1>ASS</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A119:F119">
+      <formula1>ISTORIKO_SYM</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A78:F78">
+      <formula1>metadosi</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="91" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="5" manualBreakCount="5">
     <brk id="18" max="16383" man="1"/>
-    <brk id="38" max="16383" man="1"/>
-    <brk id="48" max="16383" man="1"/>
-    <brk id="68" max="16383" man="1"/>
-    <brk id="97" max="6" man="1"/>
+    <brk id="40" max="16383" man="1"/>
+    <brk id="69" max="16383" man="1"/>
+    <brk id="98" max="16383" man="1"/>
+    <brk id="128" max="16383" man="1"/>
   </rowBreaks>
   <drawing r:id="rId2"/>
 </worksheet>
@@ -4284,10 +4288,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="33">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="232" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="220"/>
+      <c r="B1" s="232"/>
     </row>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="25" t="s">
@@ -4369,10 +4373,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="33">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="232" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="220"/>
+      <c r="B1" s="232"/>
     </row>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="25" t="s">
@@ -4454,11 +4458,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33">
-      <c r="A1" s="227" t="s">
+      <c r="A1" s="239" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="227"/>
-      <c r="C1" s="227"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
     </row>
     <row r="2" spans="1:3" ht="92.25" customHeight="1">
       <c r="A2" s="21" t="s">
@@ -4472,7 +4476,7 @@
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="200" t="str">
+      <c r="A3" s="183" t="str">
         <f>IF('Γ2 ΙΣΤΟΡΙΚΟ ΣΥΜΜΟΡΦΩΣΗΣ'!B8="-",'Δ2 ΑΡΧΙΚΗ ΑΞΙΟΛΟΓΗΣΗ'!A3:A5+'Γ1 ΑΠΟΤΕΛΕΣΜΑ ΕΛΕΓΧΟΥ'!B8,"-")</f>
         <v>-</v>
       </c>
@@ -4484,7 +4488,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="200"/>
+      <c r="A4" s="183"/>
       <c r="B4" s="19" t="s">
         <v>90</v>
       </c>
@@ -4493,7 +4497,7 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="200"/>
+      <c r="A5" s="183"/>
       <c r="B5" s="12" t="s">
         <v>91</v>
       </c>
@@ -4509,11 +4513,11 @@
       <c r="A7" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="235" t="str">
+      <c r="B7" s="247" t="str">
         <f>IF($A$3&lt;=19,$C$3,IF($A$3&lt;=39,$C$4,IF($A$3="-","-",C$5)))</f>
         <v>-</v>
       </c>
-      <c r="C7" s="236"/>
+      <c r="C7" s="248"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4537,11 +4541,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="250" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="238"/>
-      <c r="C1" s="238"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
       <c r="D1" s="20"/>
     </row>
     <row r="2" spans="1:4" ht="92.25" customHeight="1">
@@ -4556,7 +4560,7 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="200">
+      <c r="A3" s="183">
         <f>IF('Γ2 ΙΣΤΟΡΙΚΟ ΣΥΜΜΟΡΦΩΣΗΣ'!B8&lt;&gt;"-",SUM('Β1 ΤΥΠΟΣ ΠΛΗΡΟΤΗΤΑΣ'!C10+'B2 ΡΥΘΜΟΣ ΑΝΑΠΤΥΞΗΣ ΠΥΡΚΑΓΙΑΣ'!D8,'B3 ΠΛΗΘΟΣ ΧΡΗΣΤΩΝ'!C8+'Β4 ΚΤΙΡΙΑΚΗ ΠΟΛΥΠΛΟΚΟΤΗΤΑ'!C7+'Β5 ΜΕΤΑΔΟΣΗ ΠΥΡΚΑΓΙΑΣ'!C7+'Γ1 ΑΠΟΤΕΛΕΣΜΑ ΕΛΕΓΧΟΥ'!B8+'Γ2 ΙΣΤΟΡΙΚΟ ΣΥΜΜΟΡΦΩΣΗΣ'!B8),"-")</f>
         <v>52</v>
       </c>
@@ -4568,7 +4572,7 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="200"/>
+      <c r="A4" s="183"/>
       <c r="B4" s="19" t="s">
         <v>87</v>
       </c>
@@ -4577,7 +4581,7 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="200"/>
+      <c r="A5" s="183"/>
       <c r="B5" s="12" t="s">
         <v>88</v>
       </c>
@@ -4593,11 +4597,11 @@
       <c r="A7" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="237" t="str">
+      <c r="B7" s="249" t="str">
         <f>IF(A3="-","-",IF($A$3&lt;=21,$C$3,IF($A$3&lt;=43,$C$4,$C$5)))</f>
         <v>Υψηλό</v>
       </c>
-      <c r="C7" s="237"/>
+      <c r="C7" s="249"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4623,82 +4627,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="212" t="s">
+      <c r="A1" s="224" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="212"/>
-      <c r="C1" s="212"/>
-      <c r="D1" s="212"/>
+      <c r="B1" s="224"/>
+      <c r="C1" s="224"/>
+      <c r="D1" s="224"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="156" t="s">
+      <c r="B2" s="169" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="158"/>
+      <c r="C2" s="170"/>
+      <c r="D2" s="171"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="213" t="s">
+      <c r="B3" s="225" t="s">
         <v>104</v>
       </c>
-      <c r="C3" s="214"/>
-      <c r="D3" s="215"/>
+      <c r="C3" s="226"/>
+      <c r="D3" s="227"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="216" t="s">
+      <c r="B4" s="228" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="217"/>
-      <c r="D4" s="218"/>
+      <c r="C4" s="229"/>
+      <c r="D4" s="230"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="213" t="s">
+      <c r="B5" s="225" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="214"/>
-      <c r="D5" s="215"/>
+      <c r="C5" s="226"/>
+      <c r="D5" s="227"/>
     </row>
     <row r="6" spans="1:4" ht="15.75">
-      <c r="A6" s="154" t="s">
+      <c r="A6" s="166" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="154"/>
-      <c r="C6" s="154"/>
-      <c r="D6" s="154"/>
+      <c r="B6" s="166"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
     </row>
     <row r="7" spans="1:4" ht="54" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="206" t="s">
+      <c r="B7" s="218" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="207"/>
-      <c r="D7" s="208"/>
+      <c r="C7" s="219"/>
+      <c r="D7" s="220"/>
     </row>
     <row r="8" spans="1:4" ht="88.5" customHeight="1">
       <c r="A8" s="36" t="str">
         <f>IF('Δ3 ΤΕΛΙΚΟ ΕΠΙΠΕΔΟ ΧΩΡΙΣ ΙΣΤΟΡΙΚ'!A3&lt;&gt;"-",'Δ3 ΤΕΛΙΚΟ ΕΠΙΠΕΔΟ ΧΩΡΙΣ ΙΣΤΟΡΙΚ'!B7,'Δ3 ΤΕΛΙΚΟ ΕΠΙΠΕΔΟ ΜΕ ΙΣΤΟΡΙΚΟ'!B7)</f>
         <v>Υψηλό</v>
       </c>
-      <c r="B8" s="239" t="str">
+      <c r="B8" s="251" t="str">
         <f>IF(A8=A3,B3,IF(A8=A4,B4,B5))</f>
         <v>Κάθε 12 μήνες</v>
       </c>
-      <c r="C8" s="240"/>
-      <c r="D8" s="241"/>
+      <c r="C8" s="252"/>
+      <c r="D8" s="253"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="20" t="s">
@@ -4737,82 +4741,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="212" t="s">
+      <c r="A1" s="224" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="212"/>
-      <c r="C1" s="212"/>
-      <c r="D1" s="212"/>
+      <c r="B1" s="224"/>
+      <c r="C1" s="224"/>
+      <c r="D1" s="224"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="156" t="s">
+      <c r="B2" s="169" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="158"/>
+      <c r="C2" s="170"/>
+      <c r="D2" s="171"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="213" t="s">
+      <c r="B3" s="225" t="s">
         <v>132</v>
       </c>
-      <c r="C3" s="214"/>
-      <c r="D3" s="215"/>
+      <c r="C3" s="226"/>
+      <c r="D3" s="227"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="216" t="s">
+      <c r="B4" s="228" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="217"/>
-      <c r="D4" s="218"/>
+      <c r="C4" s="229"/>
+      <c r="D4" s="230"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="213" t="s">
+      <c r="B5" s="225" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="214"/>
-      <c r="D5" s="215"/>
+      <c r="C5" s="226"/>
+      <c r="D5" s="227"/>
     </row>
     <row r="6" spans="1:4" ht="15.75">
-      <c r="A6" s="154" t="s">
+      <c r="A6" s="166" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="154"/>
-      <c r="C6" s="154"/>
-      <c r="D6" s="154"/>
+      <c r="B6" s="166"/>
+      <c r="C6" s="166"/>
+      <c r="D6" s="166"/>
     </row>
     <row r="7" spans="1:4" ht="36">
       <c r="A7" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="206" t="s">
+      <c r="B7" s="218" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="207"/>
-      <c r="D7" s="208"/>
+      <c r="C7" s="219"/>
+      <c r="D7" s="220"/>
     </row>
     <row r="8" spans="1:4" ht="84" customHeight="1">
       <c r="A8" s="36" t="str">
         <f>'Δ2 ΑΡΧΙΚΗ ΑΞΙΟΛΟΓΗΣΗ'!B6</f>
         <v>Υψηλό</v>
       </c>
-      <c r="B8" s="209" t="str">
+      <c r="B8" s="221" t="str">
         <f>IF(A8=A3,B3,IF(A8=A4,B4,B5))</f>
         <v>Κάθε 12 μήνες</v>
       </c>
-      <c r="C8" s="210"/>
-      <c r="D8" s="211"/>
+      <c r="C8" s="222"/>
+      <c r="D8" s="223"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -4849,11 +4853,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="232" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="220"/>
-      <c r="C1" s="220"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="232"/>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1">
       <c r="A2" s="7" t="s">
@@ -4933,19 +4937,19 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="18">
-      <c r="A9" s="161" t="s">
+      <c r="A9" s="187" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="161"/>
+      <c r="B9" s="187"/>
       <c r="C9" s="10" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="33.75">
-      <c r="A10" s="219" t="s">
+      <c r="A10" s="231" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="219"/>
+      <c r="B10" s="231"/>
       <c r="C10" s="9">
         <f>IF($A$10=$A$3,$C$3,IF($A$10=$A$4,$C$4,IF($A$10=$A$5,$C$5,IF($A$10=$A$6,$C$6,IF($A$10=$A$7,$C$7,$C$8)))))</f>
         <v>16</v>
@@ -4981,12 +4985,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5">
-      <c r="A1" s="212" t="s">
+      <c r="A1" s="224" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="212"/>
-      <c r="C1" s="212"/>
-      <c r="D1" s="212"/>
+      <c r="B1" s="224"/>
+      <c r="C1" s="224"/>
+      <c r="D1" s="224"/>
     </row>
     <row r="2" spans="1:4" ht="66.75" customHeight="1">
       <c r="A2" s="7" t="s">
@@ -5059,21 +5063,21 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="33.75" customHeight="1">
-      <c r="A7" s="114" t="s">
+      <c r="A7" s="125" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="115"/>
-      <c r="C7" s="116"/>
+      <c r="B7" s="126"/>
+      <c r="C7" s="127"/>
       <c r="D7" s="10" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="33.75">
-      <c r="A8" s="221">
+      <c r="A8" s="233">
         <v>4</v>
       </c>
-      <c r="B8" s="222"/>
-      <c r="C8" s="223"/>
+      <c r="B8" s="234"/>
+      <c r="C8" s="235"/>
       <c r="D8" s="37">
         <f>IF(A8=A3,D3,IF(A8=A4,D4,IF(A8=A5,D5,D6)))</f>
         <v>12</v>
@@ -5109,33 +5113,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33">
-      <c r="A1" s="227" t="s">
+      <c r="A1" s="239" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="227"/>
-      <c r="C1" s="227"/>
-      <c r="D1" s="227"/>
-      <c r="E1" s="227"/>
-      <c r="F1" s="227"/>
-      <c r="G1" s="227"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
+      <c r="D1" s="239"/>
+      <c r="E1" s="239"/>
+      <c r="F1" s="239"/>
+      <c r="G1" s="239"/>
     </row>
     <row r="2" spans="1:7" ht="51" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="117" t="s">
+      <c r="B2" s="128" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117" t="s">
+      <c r="C2" s="128"/>
+      <c r="D2" s="128" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="117"/>
+      <c r="E2" s="128"/>
+      <c r="F2" s="128"/>
+      <c r="G2" s="128"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="124">
+      <c r="A3" s="135">
         <f>SUM('Β1 ΤΥΠΟΣ ΠΛΗΡΟΤΗΤΑΣ'!C10+'B2 ΡΥΘΜΟΣ ΑΝΑΠΤΥΞΗΣ ΠΥΡΚΑΓΙΑΣ'!D8)</f>
         <v>28</v>
       </c>
@@ -5145,68 +5149,68 @@
       <c r="C3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="110" t="s">
+      <c r="D3" s="121" t="s">
         <v>124</v>
       </c>
-      <c r="E3" s="110"/>
-      <c r="F3" s="110"/>
-      <c r="G3" s="110"/>
+      <c r="E3" s="121"/>
+      <c r="F3" s="121"/>
+      <c r="G3" s="121"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="124"/>
+      <c r="A4" s="135"/>
       <c r="B4" s="12" t="s">
         <v>33</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="110" t="s">
+      <c r="D4" s="121" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="121"/>
+      <c r="G4" s="121"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="124"/>
+      <c r="A5" s="135"/>
       <c r="B5" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="110"/>
-      <c r="E5" s="110"/>
-      <c r="F5" s="110"/>
-      <c r="G5" s="110"/>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
     </row>
     <row r="6" spans="1:7" ht="33.75">
-      <c r="A6" s="226" t="s">
+      <c r="A6" s="238" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="226"/>
+      <c r="B6" s="238"/>
       <c r="C6" s="9" t="str">
         <f>IF($A$3&lt;=8,$C$3,IF($A$3&lt;=18,$C$4,$C$5))</f>
         <v>Υψηλό</v>
       </c>
-      <c r="D6" s="219" t="str">
+      <c r="D6" s="231" t="str">
         <f>IF($A$3&lt;=8,$D$3,$D$4)</f>
         <v>ΝΑΙ</v>
       </c>
-      <c r="E6" s="219"/>
-      <c r="F6" s="219"/>
-      <c r="G6" s="219"/>
+      <c r="E6" s="231"/>
+      <c r="F6" s="231"/>
+      <c r="G6" s="231"/>
     </row>
     <row r="7" spans="1:7" ht="42" customHeight="1">
-      <c r="A7" s="224" t="s">
+      <c r="A7" s="236" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="225"/>
-      <c r="C7" s="225"/>
-      <c r="D7" s="225"/>
-      <c r="E7" s="225"/>
-      <c r="F7" s="225"/>
-      <c r="G7" s="225"/>
+      <c r="B7" s="237"/>
+      <c r="C7" s="237"/>
+      <c r="D7" s="237"/>
+      <c r="E7" s="237"/>
+      <c r="F7" s="237"/>
+      <c r="G7" s="237"/>
     </row>
     <row r="9" spans="1:7" ht="66.75" customHeight="1"/>
   </sheetData>
@@ -5238,11 +5242,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="34.5">
-      <c r="A1" s="228" t="s">
+      <c r="A1" s="240" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="228"/>
-      <c r="C1" s="228"/>
+      <c r="B1" s="240"/>
+      <c r="C1" s="240"/>
     </row>
     <row r="2" spans="1:3" ht="15.75">
       <c r="A2" s="15" t="s">
@@ -5300,19 +5304,19 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="60.75" customHeight="1">
-      <c r="A7" s="99" t="s">
+      <c r="A7" s="113" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="99"/>
+      <c r="B7" s="113"/>
       <c r="C7" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="33.75">
-      <c r="A8" s="219" t="s">
+      <c r="A8" s="231" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="219"/>
+      <c r="B8" s="231"/>
       <c r="C8" s="9">
         <f>IF($A$8=$A$3,$C$3,IF($A$8=$A$4,$C$4,IF($A$8=$A$5,$C$5,$C$6)))</f>
         <v>6</v>
@@ -5346,11 +5350,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="232" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="220"/>
-      <c r="C1" s="220"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="232"/>
     </row>
     <row r="2" spans="1:3" ht="15.75">
       <c r="A2" s="15" t="s">
@@ -5397,19 +5401,19 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" customHeight="1">
-      <c r="A6" s="229" t="s">
+      <c r="A6" s="241" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="229"/>
+      <c r="B6" s="241"/>
       <c r="C6" s="17" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="33.75">
-      <c r="A7" s="219" t="s">
+      <c r="A7" s="231" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="219"/>
+      <c r="B7" s="231"/>
       <c r="C7" s="9">
         <f>IF($A$7=$A$3,$C$3,IF($A$7=$A$4,$C$4,$C$5))</f>
         <v>0</v>
@@ -5444,12 +5448,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="232" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="220"/>
-      <c r="C1" s="220"/>
-      <c r="D1" s="220"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="232"/>
+      <c r="D1" s="232"/>
     </row>
     <row r="2" spans="1:4" ht="15.75">
       <c r="A2" s="15" t="s">
@@ -5508,25 +5512,25 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="51.75" customHeight="1">
-      <c r="A6" s="151" t="s">
+      <c r="A6" s="164" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="151"/>
-      <c r="C6" s="230" t="s">
+      <c r="B6" s="164"/>
+      <c r="C6" s="242" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="231"/>
+      <c r="D6" s="243"/>
     </row>
     <row r="7" spans="1:4" ht="33.75">
-      <c r="A7" s="219">
+      <c r="A7" s="231">
         <v>1</v>
       </c>
-      <c r="B7" s="219"/>
-      <c r="C7" s="221">
+      <c r="B7" s="231"/>
+      <c r="C7" s="233">
         <f>IF($A$7=$A$3,$D$3,IF($A$7=$A$4,$D$4,$D$5))</f>
         <v>0</v>
       </c>
-      <c r="D7" s="223"/>
+      <c r="D7" s="235"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5558,11 +5562,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33">
-      <c r="A1" s="232" t="s">
+      <c r="A1" s="244" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="232"/>
-      <c r="C1" s="232"/>
+      <c r="B1" s="244"/>
+      <c r="C1" s="244"/>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
       <c r="F1" s="18"/>
@@ -5572,13 +5576,13 @@
       <c r="A2" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="233" t="s">
+      <c r="B2" s="245" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="233"/>
+      <c r="C2" s="245"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="234">
+      <c r="A3" s="246">
         <f>SUM('Β1 ΤΥΠΟΣ ΠΛΗΡΟΤΗΤΑΣ'!C10+'B2 ΡΥΘΜΟΣ ΑΝΑΠΤΥΞΗΣ ΠΥΡΚΑΓΙΑΣ'!D8,'B3 ΠΛΗΘΟΣ ΧΡΗΣΤΩΝ'!C8+'Β4 ΚΤΙΡΙΑΚΗ ΠΟΛΥΠΛΟΚΟΤΗΤΑ'!C7+'Β5 ΜΕΤΑΔΟΣΗ ΠΥΡΚΑΓΙΑΣ'!C7)</f>
         <v>34</v>
       </c>
@@ -5590,7 +5594,7 @@
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="234"/>
+      <c r="A4" s="246"/>
       <c r="B4" s="19" t="s">
         <v>69</v>
       </c>
@@ -5599,7 +5603,7 @@
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="234"/>
+      <c r="A5" s="246"/>
       <c r="B5" s="12" t="s">
         <v>70</v>
       </c>
@@ -5611,11 +5615,11 @@
       <c r="A6" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="221" t="str">
+      <c r="B6" s="233" t="str">
         <f>IF($A$3&lt;=14,$C$3,IF($A$3&lt;=30,$C$4,C$5))</f>
         <v>Υψηλό</v>
       </c>
-      <c r="C6" s="223"/>
+      <c r="C6" s="235"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>